<commit_message>
Rebuild 2024-2023 statements from Kertas Kerja Lengkap and audit draft
Use Draft Report BJS 2025 for 2024 (restated) figures and cross-check 2023
against the consolidated worksheet. Cash flow now separates the gain and
proceeds on investment property sale, audited depreciation, and non-cash
right-of-use additions.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjSdhC6QBwRWgLXFLCYfr
</commit_message>
<xml_diff>
--- a/output/Laporan_Keuangan_PT_Bukit_Jaya_Semesta_2024_2023.xlsx
+++ b/output/Laporan_Keuangan_PT_Bukit_Jaya_Semesta_2024_2023.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="27">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -162,8 +162,17 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF0000FF"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -337,7 +346,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4"/>
     <xf numFmtId="41" fontId="8" fillId="0" borderId="4"/>
   </cellStyleXfs>
-  <cellXfs count="89">
+  <cellXfs count="91">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -498,7 +507,7 @@
     <xf numFmtId="41" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="22" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="24" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="41" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -507,8 +516,12 @@
     <xf numFmtId="41" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="41" fontId="23" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -521,13 +534,13 @@
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="41" fontId="8" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="41" fontId="8" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -909,7 +922,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -918,7 +931,7 @@
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="3" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="62" customWidth="1" min="8" max="8"/>
+    <col width="64" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1040,16 +1053,16 @@
     <row r="10">
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Beban Penyusutan Aset Tetap</t>
+          <t xml:space="preserve">  Beban Penyusutan &amp; Amortisasi</t>
         </is>
       </c>
       <c r="C10" s="64">
-        <f>'Neraca (Balance Sheet)'!D23</f>
+        <f>$C$80</f>
         <v/>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Akumulasi Penyusutan</t>
+          <t>Input laporan audit (Catatan 12, 14, 23, 25)</t>
         </is>
       </c>
       <c r="G10" s="43">
@@ -1058,135 +1071,135 @@
       </c>
       <c r="H10" s="42" t="inlineStr">
         <is>
-          <t>• Penyusutan Aset Tetap</t>
+          <t>• Penyusutan &amp; Amortisasi</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Penghasilan Komprehensif Lain (non-kas)</t>
+          <t xml:space="preserve">  Laba Penjualan Properti Investasi (non-kas)</t>
         </is>
       </c>
       <c r="C11" s="64">
-        <f>'Laba Rugi (Income Statement)'!B32</f>
+        <f>-$C$73</f>
         <v/>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Laba Rugi - Total OCI</t>
+          <t>Input laporan audit - dipindah ke investasi</t>
         </is>
       </c>
       <c r="G11" s="43">
-        <f>-'Laba Rugi (Income Statement)'!B17</f>
+        <f>C11</f>
         <v/>
       </c>
       <c r="H11" s="42" t="inlineStr">
         <is>
-          <t>• Beban Keuangan (Finance Expense)</t>
+          <t>• Laba Penjualan Properti Investasi</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Penyesuaian Saldo Laba (selisih Neraca vs Laba Rugi)</t>
+          <t xml:space="preserve">  Penghasilan Komprehensif Lain (non-kas)</t>
         </is>
       </c>
       <c r="C12" s="64">
-        <f>-'Neraca (Balance Sheet)'!D66-'Laba Rugi (Income Statement)'!B45</f>
+        <f>'Laba Rugi (Income Statement)'!B32</f>
         <v/>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>Neraca Saldo Laba - Laba Komprehensif Mayoritas</t>
+          <t>Laba Rugi - Total OCI</t>
         </is>
       </c>
       <c r="G12" s="43">
-        <f>-'Laba Rugi (Income Statement)'!B16</f>
+        <f>-'Laba Rugi (Income Statement)'!B17</f>
         <v/>
       </c>
       <c r="H12" s="42" t="inlineStr">
         <is>
-          <t>• Pendapatan Bunga / Keuangan</t>
+          <t>• Beban Keuangan (Finance Expense)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="10" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Penyesuaian Saldo Laba (selisih Neraca vs Laba Rugi)</t>
+        </is>
+      </c>
+      <c r="C13" s="64">
+        <f>-'Neraca (Balance Sheet)'!D66-'Laba Rugi (Income Statement)'!B45</f>
+        <v/>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>Neraca Saldo Laba - Laba Komprehensif Mayoritas</t>
+        </is>
+      </c>
+      <c r="G13" s="43">
+        <f>-'Laba Rugi (Income Statement)'!B16</f>
+        <v/>
+      </c>
+      <c r="H13" s="42" t="inlineStr">
+        <is>
+          <t>• Pendapatan Keuangan (Bunga &amp; Dividen)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="10" t="inlineStr">
+        <is>
           <t xml:space="preserve">  (Kenaikan) Penurunan Aset Pajak Tangguhan</t>
         </is>
       </c>
-      <c r="C13" s="64">
+      <c r="C14" s="64">
         <f>'Neraca (Balance Sheet)'!D30</f>
         <v/>
       </c>
-      <c r="D13" s="10" t="inlineStr">
+      <c r="D14" s="10" t="inlineStr">
         <is>
           <t>Neraca - Selisih Aset Pajak Tangguhan</t>
         </is>
       </c>
-      <c r="G13" s="43">
-        <f>C11+C12</f>
-        <v/>
-      </c>
-      <c r="H13" s="42" t="inlineStr">
+      <c r="G14" s="43">
+        <f>C12+C13</f>
+        <v/>
+      </c>
+      <c r="H14" s="42" t="inlineStr">
         <is>
           <t>• Penghasilan Komprehensif Lain &amp; Penyesuaian Saldo Laba</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="13" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="13" t="inlineStr">
         <is>
           <t>Perubahan dalam Aset dan Liabilitas Operasi:</t>
         </is>
       </c>
-      <c r="H14" s="41" t="inlineStr">
+      <c r="H15" s="41" t="inlineStr">
         <is>
           <t>Perubahan Modal Kerja:</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="10" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  (Kenaikan) Penurunan Restricted Cash</t>
-        </is>
-      </c>
-      <c r="C15" s="64">
-        <f>'Neraca (Balance Sheet)'!D9</f>
-        <v/>
-      </c>
-      <c r="D15" s="10" t="inlineStr">
-        <is>
-          <t>Neraca - Selisih Restricted Cash</t>
-        </is>
-      </c>
-      <c r="G15" s="43">
-        <f>C15</f>
-        <v/>
-      </c>
-      <c r="H15" s="42" t="inlineStr">
-        <is>
-          <t>• (Kenaikan) Penurunan Restricted Cash</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Kenaikan) Penurunan Piutang Usaha - Bersih</t>
+          <t xml:space="preserve">  (Kenaikan) Penurunan Restricted Cash</t>
         </is>
       </c>
       <c r="C16" s="64">
-        <f>'Neraca (Balance Sheet)'!D10</f>
+        <f>'Neraca (Balance Sheet)'!D9</f>
         <v/>
       </c>
       <c r="D16" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Piutang Usaha - Bersih</t>
+          <t>Neraca - Selisih Restricted Cash</t>
         </is>
       </c>
       <c r="G16" s="43">
@@ -1195,23 +1208,23 @@
       </c>
       <c r="H16" s="42" t="inlineStr">
         <is>
-          <t>• (Kenaikan) Penurunan Piutang Usaha - Bersih</t>
+          <t>• (Kenaikan) Penurunan Restricted Cash</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Kenaikan) Penurunan Piutang Lain-lain - Pihak Ketiga</t>
+          <t xml:space="preserve">  (Kenaikan) Penurunan Piutang Usaha - Bersih</t>
         </is>
       </c>
       <c r="C17" s="64">
-        <f>'Neraca (Balance Sheet)'!D11</f>
+        <f>'Neraca (Balance Sheet)'!D10</f>
         <v/>
       </c>
       <c r="D17" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Piutang Lain-lain - Pihak Ketiga</t>
+          <t>Neraca - Selisih Piutang Usaha - Bersih</t>
         </is>
       </c>
       <c r="G17" s="43">
@@ -1220,23 +1233,23 @@
       </c>
       <c r="H17" s="42" t="inlineStr">
         <is>
-          <t>• (Kenaikan) Penurunan Piutang Lain-lain - Pihak Ketiga</t>
+          <t>• (Kenaikan) Penurunan Piutang Usaha - Bersih</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Kenaikan) Penurunan Piutang Lain-lain - Pihak Berelasi</t>
+          <t xml:space="preserve">  (Kenaikan) Penurunan Piutang Lain-lain - Pihak Ketiga</t>
         </is>
       </c>
       <c r="C18" s="64">
-        <f>'Neraca (Balance Sheet)'!D12</f>
+        <f>'Neraca (Balance Sheet)'!D11</f>
         <v/>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Piutang Lain-lain - Pihak Berelasi</t>
+          <t>Neraca - Selisih Piutang Lain-lain - Pihak Ketiga</t>
         </is>
       </c>
       <c r="G18" s="43">
@@ -1245,23 +1258,23 @@
       </c>
       <c r="H18" s="42" t="inlineStr">
         <is>
-          <t>• (Kenaikan) Penurunan Piutang Lain-lain - Pihak Berelasi</t>
+          <t>• (Kenaikan) Penurunan Piutang Lain-lain - Pihak Ketiga</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Kenaikan) Penurunan Pajak Dibayar di Muka</t>
+          <t xml:space="preserve">  (Kenaikan) Penurunan Piutang Lain-lain - Pihak Berelasi</t>
         </is>
       </c>
       <c r="C19" s="64">
-        <f>'Neraca (Balance Sheet)'!D13</f>
+        <f>'Neraca (Balance Sheet)'!D12</f>
         <v/>
       </c>
       <c r="D19" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Pajak Dibayar di Muka</t>
+          <t>Neraca - Selisih Piutang Lain-lain - Pihak Berelasi</t>
         </is>
       </c>
       <c r="G19" s="43">
@@ -1270,23 +1283,23 @@
       </c>
       <c r="H19" s="42" t="inlineStr">
         <is>
-          <t>• (Kenaikan) Penurunan Pajak Dibayar di Muka</t>
+          <t>• (Kenaikan) Penurunan Piutang Lain-lain - Pihak Berelasi</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Kenaikan) Penurunan Uang Muka</t>
+          <t xml:space="preserve">  (Kenaikan) Penurunan Pajak Dibayar di Muka</t>
         </is>
       </c>
       <c r="C20" s="64">
-        <f>'Neraca (Balance Sheet)'!D14</f>
+        <f>'Neraca (Balance Sheet)'!D13</f>
         <v/>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Uang Muka</t>
+          <t>Neraca - Selisih Pajak Dibayar di Muka</t>
         </is>
       </c>
       <c r="G20" s="43">
@@ -1295,23 +1308,23 @@
       </c>
       <c r="H20" s="42" t="inlineStr">
         <is>
-          <t>• (Kenaikan) Penurunan Uang Muka</t>
+          <t>• (Kenaikan) Penurunan Pajak Dibayar di Muka</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Kenaikan) Penurunan Persediaan</t>
+          <t xml:space="preserve">  (Kenaikan) Penurunan Uang Muka</t>
         </is>
       </c>
       <c r="C21" s="64">
-        <f>'Neraca (Balance Sheet)'!D15</f>
+        <f>'Neraca (Balance Sheet)'!D14</f>
         <v/>
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Persediaan</t>
+          <t>Neraca - Selisih Uang Muka</t>
         </is>
       </c>
       <c r="G21" s="43">
@@ -1320,23 +1333,23 @@
       </c>
       <c r="H21" s="42" t="inlineStr">
         <is>
-          <t>• (Kenaikan) Penurunan Persediaan</t>
+          <t>• (Kenaikan) Penurunan Uang Muka</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Kenaikan) Penurunan Biaya Dibayar di Muka</t>
+          <t xml:space="preserve">  (Kenaikan) Penurunan Persediaan</t>
         </is>
       </c>
       <c r="C22" s="64">
-        <f>'Neraca (Balance Sheet)'!D16</f>
+        <f>'Neraca (Balance Sheet)'!D15</f>
         <v/>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Biaya Dibayar di Muka</t>
+          <t>Neraca - Selisih Persediaan</t>
         </is>
       </c>
       <c r="G22" s="43">
@@ -1345,23 +1358,23 @@
       </c>
       <c r="H22" s="42" t="inlineStr">
         <is>
-          <t>• (Kenaikan) Penurunan Biaya Dibayar di Muka</t>
+          <t>• (Kenaikan) Penurunan Persediaan</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Kenaikan) Penurunan Persediaan Biologis</t>
+          <t xml:space="preserve">  (Kenaikan) Penurunan Biaya Dibayar di Muka</t>
         </is>
       </c>
       <c r="C23" s="64">
-        <f>'Neraca (Balance Sheet)'!D17</f>
+        <f>'Neraca (Balance Sheet)'!D16</f>
         <v/>
       </c>
       <c r="D23" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Persediaan Biologis</t>
+          <t>Neraca - Selisih Biaya Dibayar di Muka</t>
         </is>
       </c>
       <c r="G23" s="43">
@@ -1370,23 +1383,23 @@
       </c>
       <c r="H23" s="42" t="inlineStr">
         <is>
-          <t>• (Kenaikan) Penurunan Persediaan Biologis</t>
+          <t>• (Kenaikan) Penurunan Biaya Dibayar di Muka</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  (Kenaikan) Penurunan Estimasi Klaim Pajak</t>
+          <t xml:space="preserve">  (Kenaikan) Penurunan Persediaan Biologis</t>
         </is>
       </c>
       <c r="C24" s="64">
-        <f>'Neraca (Balance Sheet)'!D26</f>
+        <f>'Neraca (Balance Sheet)'!D17</f>
         <v/>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Estimasi Klaim Pajak</t>
+          <t>Neraca - Selisih Persediaan Biologis</t>
         </is>
       </c>
       <c r="G24" s="43">
@@ -1395,23 +1408,23 @@
       </c>
       <c r="H24" s="42" t="inlineStr">
         <is>
-          <t>• (Kenaikan) Penurunan Estimasi Klaim Pajak</t>
+          <t>• (Kenaikan) Penurunan Persediaan Biologis</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Kenaikan (Penurunan) Utang Usaha</t>
+          <t xml:space="preserve">  (Kenaikan) Penurunan Estimasi Klaim Pajak</t>
         </is>
       </c>
       <c r="C25" s="64">
-        <f>-'Neraca (Balance Sheet)'!D39</f>
+        <f>'Neraca (Balance Sheet)'!D26</f>
         <v/>
       </c>
       <c r="D25" s="10" t="inlineStr">
         <is>
-          <t>Neraca - ( - Selisih Utang Usaha )</t>
+          <t>Neraca - Selisih Estimasi Klaim Pajak</t>
         </is>
       </c>
       <c r="G25" s="43">
@@ -1420,23 +1433,23 @@
       </c>
       <c r="H25" s="42" t="inlineStr">
         <is>
-          <t>• Kenaikan (Penurunan) Utang Usaha</t>
+          <t>• (Kenaikan) Penurunan Estimasi Klaim Pajak</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Kenaikan (Penurunan) Utang Pajak</t>
+          <t xml:space="preserve">  Kenaikan (Penurunan) Utang Usaha</t>
         </is>
       </c>
       <c r="C26" s="64">
-        <f>-'Neraca (Balance Sheet)'!D40</f>
+        <f>-'Neraca (Balance Sheet)'!D39</f>
         <v/>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>Neraca - ( - Selisih Utang Pajak )</t>
+          <t>Neraca - ( - Selisih Utang Usaha )</t>
         </is>
       </c>
       <c r="G26" s="43">
@@ -1445,23 +1458,23 @@
       </c>
       <c r="H26" s="42" t="inlineStr">
         <is>
-          <t>• Kenaikan (Penurunan) Utang Pajak</t>
+          <t>• Kenaikan (Penurunan) Utang Usaha</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="B27" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Kenaikan (Penurunan) Uang Muka Penjualan</t>
+          <t xml:space="preserve">  Kenaikan (Penurunan) Utang Pajak</t>
         </is>
       </c>
       <c r="C27" s="64">
-        <f>-'Neraca (Balance Sheet)'!D41</f>
+        <f>-'Neraca (Balance Sheet)'!D40</f>
         <v/>
       </c>
       <c r="D27" s="10" t="inlineStr">
         <is>
-          <t>Neraca - ( - Selisih Uang Muka Penjualan )</t>
+          <t>Neraca - ( - Selisih Utang Pajak )</t>
         </is>
       </c>
       <c r="G27" s="43">
@@ -1470,23 +1483,23 @@
       </c>
       <c r="H27" s="42" t="inlineStr">
         <is>
-          <t>• Kenaikan (Penurunan) Uang Muka Penjualan</t>
+          <t>• Kenaikan (Penurunan) Utang Pajak</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="B28" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Kenaikan (Penurunan) Biaya Masih Harus Dibayar</t>
+          <t xml:space="preserve">  Kenaikan (Penurunan) Uang Muka Penjualan</t>
         </is>
       </c>
       <c r="C28" s="64">
-        <f>-'Neraca (Balance Sheet)'!D42</f>
+        <f>-'Neraca (Balance Sheet)'!D41</f>
         <v/>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>Neraca - ( - Selisih Biaya Masih Harus Dibayar )</t>
+          <t>Neraca - ( - Selisih Uang Muka Penjualan )</t>
         </is>
       </c>
       <c r="G28" s="43">
@@ -1495,23 +1508,23 @@
       </c>
       <c r="H28" s="42" t="inlineStr">
         <is>
-          <t>• Kenaikan (Penurunan) Biaya Masih Harus Dibayar</t>
+          <t>• Kenaikan (Penurunan) Uang Muka Penjualan</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Kenaikan (Penurunan) Imbalan Kerja Jangka Pendek</t>
+          <t xml:space="preserve">  Kenaikan (Penurunan) Biaya Masih Harus Dibayar</t>
         </is>
       </c>
       <c r="C29" s="64">
-        <f>-'Neraca (Balance Sheet)'!D43</f>
+        <f>-'Neraca (Balance Sheet)'!D42</f>
         <v/>
       </c>
       <c r="D29" s="10" t="inlineStr">
         <is>
-          <t>Neraca - ( - Selisih Imbalan Kerja Jangka Pendek )</t>
+          <t>Neraca - ( - Selisih Biaya Masih Harus Dibayar )</t>
         </is>
       </c>
       <c r="G29" s="43">
@@ -1520,23 +1533,23 @@
       </c>
       <c r="H29" s="42" t="inlineStr">
         <is>
-          <t>• Kenaikan (Penurunan) Imbalan Kerja Jangka Pendek</t>
+          <t>• Kenaikan (Penurunan) Biaya Masih Harus Dibayar</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Kenaikan (Penurunan) Utang Lain-lain - Pihak Ketiga</t>
+          <t xml:space="preserve">  Kenaikan (Penurunan) Imbalan Kerja Jangka Pendek</t>
         </is>
       </c>
       <c r="C30" s="64">
-        <f>-'Neraca (Balance Sheet)'!D44</f>
+        <f>-'Neraca (Balance Sheet)'!D43</f>
         <v/>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Neraca - ( - Selisih Utang Lain-lain - Pihak Ketiga )</t>
+          <t>Neraca - ( - Selisih Imbalan Kerja Jangka Pendek )</t>
         </is>
       </c>
       <c r="G30" s="43">
@@ -1545,23 +1558,23 @@
       </c>
       <c r="H30" s="42" t="inlineStr">
         <is>
-          <t>• Kenaikan (Penurunan) Utang Lain-lain - Pihak Ketiga</t>
+          <t>• Kenaikan (Penurunan) Imbalan Kerja Jangka Pendek</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Kenaikan (Penurunan) Utang Lain-lain - Pihak Berelasi</t>
+          <t xml:space="preserve">  Kenaikan (Penurunan) Utang Lain-lain - Pihak Ketiga</t>
         </is>
       </c>
       <c r="C31" s="64">
-        <f>-'Neraca (Balance Sheet)'!D45</f>
+        <f>-'Neraca (Balance Sheet)'!D44</f>
         <v/>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Neraca - ( - Selisih Utang Lain-lain - Pihak Berelasi )</t>
+          <t>Neraca - ( - Selisih Utang Lain-lain - Pihak Ketiga )</t>
         </is>
       </c>
       <c r="G31" s="43">
@@ -1570,23 +1583,23 @@
       </c>
       <c r="H31" s="42" t="inlineStr">
         <is>
-          <t>• Kenaikan (Penurunan) Utang Lain-lain - Pihak Berelasi</t>
+          <t>• Kenaikan (Penurunan) Utang Lain-lain - Pihak Ketiga</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Kenaikan (Penurunan) Imbalan Kerja Karyawan Jangka Panjang</t>
+          <t xml:space="preserve">  Kenaikan (Penurunan) Utang Lain-lain - Pihak Berelasi</t>
         </is>
       </c>
       <c r="C32" s="64">
-        <f>-'Neraca (Balance Sheet)'!D51</f>
+        <f>-'Neraca (Balance Sheet)'!D45</f>
         <v/>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>Neraca - ( - Selisih Imbalan Kerja Karyawan Jangka Panjang )</t>
+          <t>Neraca - ( - Selisih Utang Lain-lain - Pihak Berelasi )</t>
         </is>
       </c>
       <c r="G32" s="43">
@@ -1595,170 +1608,170 @@
       </c>
       <c r="H32" s="42" t="inlineStr">
         <is>
+          <t>• Kenaikan (Penurunan) Utang Lain-lain - Pihak Berelasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Kenaikan (Penurunan) Imbalan Kerja Karyawan Jangka Panjang</t>
+        </is>
+      </c>
+      <c r="C33" s="64">
+        <f>-'Neraca (Balance Sheet)'!D51</f>
+        <v/>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t>Neraca - ( - Selisih Imbalan Kerja Karyawan Jangka Panjang )</t>
+        </is>
+      </c>
+      <c r="G33" s="43">
+        <f>C33</f>
+        <v/>
+      </c>
+      <c r="H33" s="42" t="inlineStr">
+        <is>
           <t>• Kenaikan (Penurunan) Imbalan Kerja Karyawan Jangka Panjang</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="16" t="n"/>
-      <c r="B33" s="16" t="inlineStr">
-        <is>
-          <t>Kas Bersih Diperoleh dari Aktivitas Operasi</t>
-        </is>
-      </c>
-      <c r="C33" s="65">
-        <f>SUM(C8,C10,C11,C12,C13,C15,C16,C17,C18,C19,C20,C21,C22,C23,C24,C25,C26,C27,C28,C29,C30,C31,C32)</f>
-        <v/>
-      </c>
-      <c r="D33" s="16" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="16" t="n"/>
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>Kas Bersih Diperoleh dari (Digunakan untuk) Aktivitas Operasi</t>
+        </is>
+      </c>
+      <c r="C34" s="65">
+        <f>SUM(C8,C10,C11,C12,C13,C14,C16,C17,C18,C19,C20,C21,C22,C23,C24,C25,C26,C27,C28,C29,C30,C31,C32,C33)</f>
+        <v/>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
         <is>
           <t>Total Arus Kas Operasi</t>
         </is>
       </c>
-      <c r="G33" s="43">
+      <c r="G34" s="43">
         <f>'Laba Rugi (Income Statement)'!B25</f>
         <v/>
       </c>
-      <c r="H33" s="42" t="inlineStr">
+      <c r="H34" s="42" t="inlineStr">
         <is>
           <t>• Beban Pajak Penghasilan (Kini &amp; Tangguhan)</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="G34" s="43">
-        <f>C13</f>
-        <v/>
-      </c>
-      <c r="H34" s="42" t="inlineStr">
+    <row r="35">
+      <c r="G35" s="43">
+        <f>C14</f>
+        <v/>
+      </c>
+      <c r="H35" s="42" t="inlineStr">
         <is>
           <t>• (Kenaikan) Penurunan Aset Pajak Tangguhan</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="7" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr">
+      <c r="B36" s="7" t="inlineStr">
         <is>
           <t>ARUS KAS DARI AKTIVITAS INVESTASI</t>
         </is>
       </c>
-      <c r="C35" s="7" t="n"/>
-      <c r="D35" s="7" t="n"/>
-      <c r="G35" s="43">
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="7" t="n"/>
+      <c r="G36" s="43">
         <f>'Laba Rugi (Income Statement)'!B16</f>
         <v/>
       </c>
-      <c r="H35" s="42" t="inlineStr">
-        <is>
-          <t>• Penerimaan Pendapatan Bunga / Keuangan</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Perolehan Aset Tetap (Harga Perolehan)</t>
-        </is>
-      </c>
-      <c r="C36" s="64">
-        <f>'Neraca (Balance Sheet)'!D22</f>
-        <v/>
-      </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t>Neraca - Selisih Harga Perolehan Aset Tetap</t>
-        </is>
-      </c>
-      <c r="G36" s="66">
-        <f>SUM(G8,G10,G11,G12,G13,G15,G16,G17,G18,G19,G20,G21,G22,G23,G24,G25,G26,G27,G28,G29,G30,G31,G32,G33,G34,G35)</f>
-        <v/>
-      </c>
-      <c r="H36" s="41" t="inlineStr">
-        <is>
-          <t>Kas Bersih Diperoleh dari Aktivitas Operasi</t>
+      <c r="H36" s="42" t="inlineStr">
+        <is>
+          <t>• Penerimaan Pendapatan Keuangan (Bunga &amp; Dividen)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Uang Muka Pembelian Aset Tetap</t>
+          <t>Penerimaan Penjualan Properti Investasi</t>
         </is>
       </c>
       <c r="C37" s="64">
-        <f>'Neraca (Balance Sheet)'!D25</f>
+        <f>$C$74</f>
         <v/>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Uang Muka Pembelian AT</t>
+          <t>Input laporan audit</t>
+        </is>
+      </c>
+      <c r="G37" s="66">
+        <f>SUM(G8,G10,G11,G12,G13,G14,G16,G17,G18,G19,G20,G21,G22,G23,G24,G25,G26,G27,G28,G29,G30,G31,G32,G33,G34,G35,G36)</f>
+        <v/>
+      </c>
+      <c r="H37" s="41" t="inlineStr">
+        <is>
+          <t>Kas Bersih Diperoleh dari (Digunakan untuk) Aktivitas Operasi</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Penambahan Tanaman Belum Menghasilkan</t>
+          <t>Perolehan Aset Tetap, Properti Investasi &amp; Aset Tak Berwujud</t>
         </is>
       </c>
       <c r="C38" s="64">
-        <f>'Neraca (Balance Sheet)'!D31</f>
+        <f>'Neraca (Balance Sheet)'!D24-$C$80-($C$74-$C$73)+$C$79</f>
         <v/>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih TBM Bibit Durian</t>
-        </is>
-      </c>
-      <c r="H38" s="41" t="inlineStr">
-        <is>
-          <t>2. ARUS KAS DARI AKTIVITAS INVESTASI</t>
+          <t>Neraca - Selisih Nilai Buku - Penyusutan - Nilai Buku Dijual + ROU non-kas</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>Penambahan HTI</t>
+          <t>Uang Muka Pembelian Aset Tetap</t>
         </is>
       </c>
       <c r="C39" s="64">
-        <f>'Neraca (Balance Sheet)'!D29</f>
+        <f>'Neraca (Balance Sheet)'!D25</f>
         <v/>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih HTI</t>
-        </is>
-      </c>
-      <c r="G39" s="43">
-        <f>C36</f>
-        <v/>
-      </c>
-      <c r="H39" s="42" t="inlineStr">
-        <is>
-          <t>• Perolehan Aset Tetap (Harga Perolehan)</t>
+          <t>Neraca - Selisih Uang Muka Pembelian AT</t>
+        </is>
+      </c>
+      <c r="H39" s="41" t="inlineStr">
+        <is>
+          <t>2. ARUS KAS DARI AKTIVITAS INVESTASI</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>Pembelian / Penambahan Aset Lainnya</t>
+          <t>Penambahan Tanaman Belum Menghasilkan / Goodwill</t>
         </is>
       </c>
       <c r="C40" s="64">
-        <f>'Neraca (Balance Sheet)'!D32</f>
+        <f>'Neraca (Balance Sheet)'!D31</f>
         <v/>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Aset Lainnya</t>
+          <t>Neraca - Selisih TBM / Goodwill</t>
         </is>
       </c>
       <c r="G40" s="43">
@@ -1767,23 +1780,23 @@
       </c>
       <c r="H40" s="42" t="inlineStr">
         <is>
-          <t>• Uang Muka Pembelian Aset Tetap</t>
+          <t>• Penerimaan Penjualan Properti Investasi</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Piutang Pihak Berelasi (Jangka Panjang)</t>
+          <t>Penambahan HTI</t>
         </is>
       </c>
       <c r="C41" s="64">
-        <f>'Neraca (Balance Sheet)'!D27</f>
+        <f>'Neraca (Balance Sheet)'!D29</f>
         <v/>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Piutang Pihak Berelasi</t>
+          <t>Neraca - Selisih HTI</t>
         </is>
       </c>
       <c r="G41" s="43">
@@ -1792,23 +1805,23 @@
       </c>
       <c r="H41" s="42" t="inlineStr">
         <is>
-          <t>• Penambahan Tanaman Belum Menghasilkan</t>
+          <t>• Perolehan Aset Tetap, Properti Investasi &amp; Aset Tak Berwujud</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>Penambahan Investasi (setelah eliminasi laba belum terealisasi)</t>
+          <t>Pembelian / Penambahan Aset Lainnya (Uang Jaminan)</t>
         </is>
       </c>
       <c r="C42" s="64">
-        <f>'Neraca (Balance Sheet)'!D28-'Neraca (Balance Sheet)'!D60</f>
+        <f>'Neraca (Balance Sheet)'!D32</f>
         <v/>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih Investment - Selisih Laba belum terealisasi Colorpak (non-kas)</t>
+          <t>Neraca - Selisih Aset Lainnya</t>
         </is>
       </c>
       <c r="G42" s="43">
@@ -1817,24 +1830,23 @@
       </c>
       <c r="H42" s="42" t="inlineStr">
         <is>
-          <t>• Penambahan HTI</t>
+          <t>• Uang Muka Pembelian Aset Tetap</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="n"/>
-      <c r="B43" s="16" t="inlineStr">
-        <is>
-          <t>Kas Bersih Digunakan untuk Aktivitas Investasi</t>
-        </is>
-      </c>
-      <c r="C43" s="65">
-        <f>SUM(C36,C37,C38,C39,C40,C41,C42)</f>
-        <v/>
-      </c>
-      <c r="D43" s="16" t="inlineStr">
-        <is>
-          <t>Total Arus Kas Investasi</t>
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>Piutang Pihak Berelasi (Jangka Panjang)</t>
+        </is>
+      </c>
+      <c r="C43" s="64">
+        <f>'Neraca (Balance Sheet)'!D27</f>
+        <v/>
+      </c>
+      <c r="D43" s="10" t="inlineStr">
+        <is>
+          <t>Neraca - Selisih Piutang Pihak Berelasi</t>
         </is>
       </c>
       <c r="G43" s="43">
@@ -1843,169 +1855,170 @@
       </c>
       <c r="H43" s="42" t="inlineStr">
         <is>
-          <t>• Pembelian / Penambahan Aset Lainnya</t>
+          <t>• Penambahan Tanaman Belum Menghasilkan / Goodwill</t>
         </is>
       </c>
     </row>
     <row r="44">
+      <c r="B44" s="10" t="inlineStr">
+        <is>
+          <t>Penambahan Investasi (setelah eliminasi laba belum terealisasi)</t>
+        </is>
+      </c>
+      <c r="C44" s="64">
+        <f>'Neraca (Balance Sheet)'!D28-'Neraca (Balance Sheet)'!D60</f>
+        <v/>
+      </c>
+      <c r="D44" s="10" t="inlineStr">
+        <is>
+          <t>Neraca - Selisih Investment - Selisih Nilai Wajar (non-kas)</t>
+        </is>
+      </c>
       <c r="G44" s="43">
         <f>C41</f>
         <v/>
       </c>
       <c r="H44" s="42" t="inlineStr">
         <is>
-          <t>• Piutang Pihak Berelasi (Jangka Panjang)</t>
+          <t>• Penambahan HTI</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="7" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>ARUS KAS DARI AKTIVITAS PENDANAAN</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="n"/>
-      <c r="D45" s="7" t="n"/>
+      <c r="A45" s="16" t="n"/>
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>Kas Bersih Diperoleh dari (Digunakan untuk) Aktivitas Investasi</t>
+        </is>
+      </c>
+      <c r="C45" s="65">
+        <f>SUM(C37,C38,C39,C40,C41,C42,C43,C44)</f>
+        <v/>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>Total Arus Kas Investasi</t>
+        </is>
+      </c>
       <c r="G45" s="43">
         <f>C42</f>
         <v/>
       </c>
       <c r="H45" s="42" t="inlineStr">
         <is>
+          <t>• Pembelian / Penambahan Aset Lainnya (Uang Jaminan)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="G46" s="43">
+        <f>C43</f>
+        <v/>
+      </c>
+      <c r="H46" s="42" t="inlineStr">
+        <is>
+          <t>• Piutang Pihak Berelasi (Jangka Panjang)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>ARUS KAS DARI AKTIVITAS PENDANAAN</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="n"/>
+      <c r="D47" s="7" t="n"/>
+      <c r="G47" s="43">
+        <f>C44</f>
+        <v/>
+      </c>
+      <c r="H47" s="42" t="inlineStr">
+        <is>
           <t>• Penambahan Investasi (setelah eliminasi laba belum terealisasi)</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="B46" s="10" t="inlineStr">
-        <is>
-          <t>Kenaikan (Penurunan) Utang Bank Jangka Pendek</t>
-        </is>
-      </c>
-      <c r="C46" s="64">
-        <f>-'Neraca (Balance Sheet)'!D38</f>
-        <v/>
-      </c>
-      <c r="D46" s="10" t="inlineStr">
-        <is>
-          <t>Neraca - ( - Selisih Utang Bank JP )</t>
-        </is>
-      </c>
-      <c r="G46" s="66">
-        <f>SUM(G39,G40,G41,G42,G43,G44,G45)</f>
-        <v/>
-      </c>
-      <c r="H46" s="41" t="inlineStr">
-        <is>
-          <t>Kas Bersih Digunakan untuk Aktivitas Investasi</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t>Kenaikan (Penurunan) Utang Bank Jangka Panjang</t>
-        </is>
-      </c>
-      <c r="C47" s="64">
-        <f>-'Neraca (Balance Sheet)'!D52</f>
-        <v/>
-      </c>
-      <c r="D47" s="10" t="inlineStr">
-        <is>
-          <t>Neraca - ( - Selisih Utang Bank Panjang )</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="B48" s="10" t="inlineStr">
         <is>
-          <t>Kenaikan (Penurunan) Utang Pihak Berelasi Jangka Pendek</t>
+          <t>Kenaikan (Penurunan) Utang Bank Jangka Pendek</t>
         </is>
       </c>
       <c r="C48" s="64">
-        <f>-'Neraca (Balance Sheet)'!D46</f>
+        <f>-'Neraca (Balance Sheet)'!D38</f>
         <v/>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>Neraca - ( - Selisih Utang Berelasi JP )</t>
-        </is>
+          <t>Neraca - ( - Selisih Utang Bank JP )</t>
+        </is>
+      </c>
+      <c r="G48" s="66">
+        <f>SUM(G40,G41,G42,G43,G44,G45,G46,G47)</f>
+        <v/>
       </c>
       <c r="H48" s="41" t="inlineStr">
         <is>
-          <t>3. ARUS KAS DARI AKTIVITAS PENDANAAN</t>
+          <t>Kas Bersih Diperoleh dari (Digunakan untuk) Aktivitas Investasi</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="10" t="inlineStr">
         <is>
-          <t>Pembayaran Utang Pihak Berelasi Jangka Panjang</t>
+          <t>Kenaikan (Penurunan) Utang Bank Jangka Panjang</t>
         </is>
       </c>
       <c r="C49" s="64">
-        <f>-'Neraca (Balance Sheet)'!D53</f>
+        <f>-'Neraca (Balance Sheet)'!D52</f>
         <v/>
       </c>
       <c r="D49" s="10" t="inlineStr">
         <is>
-          <t>Neraca - ( - Selisih Utang Berelasi Panjang )</t>
-        </is>
-      </c>
-      <c r="G49" s="43">
-        <f>C46</f>
-        <v/>
-      </c>
-      <c r="H49" s="42" t="inlineStr">
-        <is>
-          <t>• Kenaikan (Penurunan) Utang Bank Jangka Pendek</t>
+          <t>Neraca - ( - Selisih Utang Bank Panjang )</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="10" t="inlineStr">
         <is>
-          <t>Pembayaran Liabilitas Sewa</t>
+          <t>Kenaikan (Penurunan) Utang Pihak Berelasi Jangka Pendek</t>
         </is>
       </c>
       <c r="C50" s="64">
-        <f>-('Neraca (Balance Sheet)'!D47+'Neraca (Balance Sheet)'!D54)</f>
+        <f>-'Neraca (Balance Sheet)'!D46</f>
         <v/>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Total Selisih Liabilitas Sewa</t>
-        </is>
-      </c>
-      <c r="G50" s="43">
-        <f>C47</f>
-        <v/>
-      </c>
-      <c r="H50" s="42" t="inlineStr">
-        <is>
-          <t>• Kenaikan (Penurunan) Utang Bank Jangka Panjang</t>
+          <t>Neraca - ( - Selisih Utang Berelasi JP )</t>
+        </is>
+      </c>
+      <c r="H50" s="41" t="inlineStr">
+        <is>
+          <t>3. ARUS KAS DARI AKTIVITAS PENDANAAN</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="B51" s="10" t="inlineStr">
         <is>
-          <t>Setoran Modal / Tambahan Modal Disetor</t>
+          <t>Pembayaran Utang Pihak Berelasi Jangka Panjang</t>
         </is>
       </c>
       <c r="C51" s="64">
-        <f>-('Neraca (Balance Sheet)'!D59+'Neraca (Balance Sheet)'!D61)</f>
+        <f>-'Neraca (Balance Sheet)'!D53</f>
         <v/>
       </c>
       <c r="D51" s="10" t="inlineStr">
         <is>
-          <t>Neraca - ( - Selisih Modal &amp; Tambahan Modal )</t>
+          <t>Neraca - ( - Selisih Utang Berelasi Panjang )</t>
         </is>
       </c>
       <c r="G51" s="43">
@@ -2014,23 +2027,23 @@
       </c>
       <c r="H51" s="42" t="inlineStr">
         <is>
-          <t>• Kenaikan (Penurunan) Utang Pihak Berelasi Jangka Pendek</t>
+          <t>• Kenaikan (Penurunan) Utang Bank Jangka Pendek</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>Kenaikan Akun Stress (Ekuitas Lainnya)</t>
+          <t>Pembayaran Pokok Liabilitas Sewa</t>
         </is>
       </c>
       <c r="C52" s="64">
-        <f>-'Neraca (Balance Sheet)'!D62</f>
+        <f>-('Neraca (Balance Sheet)'!D47+'Neraca (Balance Sheet)'!D54)-$C$79</f>
         <v/>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>Neraca - ( - Selisih Stress )</t>
+          <t>Neraca - Selisih Liabilitas Sewa - Penambahan ROU non-kas</t>
         </is>
       </c>
       <c r="G52" s="43">
@@ -2039,23 +2052,23 @@
       </c>
       <c r="H52" s="42" t="inlineStr">
         <is>
-          <t>• Pembayaran Utang Pihak Berelasi Jangka Panjang</t>
+          <t>• Kenaikan (Penurunan) Utang Bank Jangka Panjang</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="B53" s="10" t="inlineStr">
         <is>
-          <t>Penerimaan Setoran / Kenaikan NCI Net (di luar bagian laba NCI)</t>
+          <t>Setoran Modal / Tambahan Modal Disetor</t>
         </is>
       </c>
       <c r="C53" s="64">
-        <f>-'Neraca (Balance Sheet)'!D67-'Laba Rugi (Income Statement)'!B36-'Laba Rugi (Income Statement)'!B43</f>
+        <f>-('Neraca (Balance Sheet)'!D59+'Neraca (Balance Sheet)'!D61)</f>
         <v/>
       </c>
       <c r="D53" s="10" t="inlineStr">
         <is>
-          <t>Neraca - Selisih NCI dikurangi NCI atas Laba &amp; OCI</t>
+          <t>Neraca - ( - Selisih Modal &amp; Tambahan Modal )</t>
         </is>
       </c>
       <c r="G53" s="43">
@@ -2064,24 +2077,23 @@
       </c>
       <c r="H53" s="42" t="inlineStr">
         <is>
-          <t>• Pembayaran Liabilitas Sewa</t>
+          <t>• Kenaikan (Penurunan) Utang Pihak Berelasi Jangka Pendek</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="16" t="n"/>
-      <c r="B54" s="16" t="inlineStr">
-        <is>
-          <t>Kas Bersih Diperoleh dari Aktivitas Pendanaan</t>
-        </is>
-      </c>
-      <c r="C54" s="65">
-        <f>SUM(C46,C47,C48,C49,C50,C51,C52,C53)</f>
-        <v/>
-      </c>
-      <c r="D54" s="16" t="inlineStr">
-        <is>
-          <t>Total Arus Kas Pendanaan</t>
+      <c r="B54" s="10" t="inlineStr">
+        <is>
+          <t>Selisih Transaksi Perubahan Saham Anak (Stress)</t>
+        </is>
+      </c>
+      <c r="C54" s="64">
+        <f>-'Neraca (Balance Sheet)'!D62</f>
+        <v/>
+      </c>
+      <c r="D54" s="10" t="inlineStr">
+        <is>
+          <t>Neraca - ( - Selisih Stress )</t>
         </is>
       </c>
       <c r="G54" s="43">
@@ -2090,35 +2102,49 @@
       </c>
       <c r="H54" s="42" t="inlineStr">
         <is>
-          <t>• Setoran Modal / Tambahan Modal Disetor</t>
+          <t>• Pembayaran Utang Pihak Berelasi Jangka Panjang</t>
         </is>
       </c>
     </row>
     <row r="55">
+      <c r="B55" s="10" t="inlineStr">
+        <is>
+          <t>Penerimaan Setoran / Kenaikan NCI Net (di luar bagian laba NCI)</t>
+        </is>
+      </c>
+      <c r="C55" s="64">
+        <f>-'Neraca (Balance Sheet)'!D67-'Laba Rugi (Income Statement)'!B36-'Laba Rugi (Income Statement)'!B43</f>
+        <v/>
+      </c>
+      <c r="D55" s="10" t="inlineStr">
+        <is>
+          <t>Neraca - Selisih NCI dikurangi NCI atas Laba &amp; OCI</t>
+        </is>
+      </c>
       <c r="G55" s="43">
         <f>C52</f>
         <v/>
       </c>
       <c r="H55" s="42" t="inlineStr">
         <is>
-          <t>• Kenaikan Akun Stress (Ekuitas Lainnya)</t>
+          <t>• Pembayaran Pokok Liabilitas Sewa</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="23" t="n"/>
-      <c r="B56" s="23" t="inlineStr">
-        <is>
-          <t>KENAIKAN (PENURUNAN) BERSIH KAS DAN SETARA KAS</t>
-        </is>
-      </c>
-      <c r="C56" s="67">
-        <f>C33+C43+C54</f>
-        <v/>
-      </c>
-      <c r="D56" s="23" t="inlineStr">
-        <is>
-          <t>Arus Kas (A + B + C)</t>
+      <c r="A56" s="16" t="n"/>
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>Kas Bersih Diperoleh dari (Digunakan untuk) Aktivitas Pendanaan</t>
+        </is>
+      </c>
+      <c r="C56" s="65">
+        <f>SUM(C48,C49,C50,C51,C52,C53,C54,C55)</f>
+        <v/>
+      </c>
+      <c r="D56" s="16" t="inlineStr">
+        <is>
+          <t>Total Arus Kas Pendanaan</t>
         </is>
       </c>
       <c r="G56" s="43">
@@ -2127,165 +2153,359 @@
       </c>
       <c r="H56" s="42" t="inlineStr">
         <is>
+          <t>• Setoran Modal / Tambahan Modal Disetor</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="G57" s="43">
+        <f>C54</f>
+        <v/>
+      </c>
+      <c r="H57" s="42" t="inlineStr">
+        <is>
+          <t>• Selisih Transaksi Perubahan Saham Anak (Stress)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="23" t="n"/>
+      <c r="B58" s="23" t="inlineStr">
+        <is>
+          <t>KENAIKAN (PENURUNAN) BERSIH KAS DAN SETARA KAS</t>
+        </is>
+      </c>
+      <c r="C58" s="67">
+        <f>C34+C45+C56</f>
+        <v/>
+      </c>
+      <c r="D58" s="23" t="inlineStr">
+        <is>
+          <t>Arus Kas (A + B + C)</t>
+        </is>
+      </c>
+      <c r="G58" s="43">
+        <f>C55</f>
+        <v/>
+      </c>
+      <c r="H58" s="42" t="inlineStr">
+        <is>
           <t>• Penerimaan Setoran / Kenaikan NCI Net (di luar bagian laba NCI)</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="B57" s="13" t="inlineStr">
+    <row r="59">
+      <c r="B59" s="13" t="inlineStr">
         <is>
           <t>KAS DAN SETARA KAS AWAL PERIODE (31-DES-2023)</t>
         </is>
       </c>
-      <c r="C57" s="65">
+      <c r="C59" s="65">
         <f>'Neraca (Balance Sheet)'!C8</f>
         <v/>
       </c>
-      <c r="D57" s="10" t="inlineStr">
+      <c r="D59" s="10" t="inlineStr">
         <is>
           <t>Neraca - Kas &amp; Setara Kas 2023</t>
         </is>
       </c>
-      <c r="G57" s="43">
+      <c r="G59" s="43">
         <f>'Laba Rugi (Income Statement)'!B17</f>
         <v/>
       </c>
-      <c r="H57" s="42" t="inlineStr">
+      <c r="H59" s="42" t="inlineStr">
         <is>
           <t>• Pembayaran Beban Keuangan / Bunga</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="16" t="n"/>
-      <c r="B58" s="16" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="16" t="n"/>
+      <c r="B60" s="16" t="inlineStr">
         <is>
           <t>KAS DAN SETARA KAS AKHIR PERIODE (31-DES-2024)</t>
         </is>
       </c>
-      <c r="C58" s="65">
-        <f>C56+C57</f>
-        <v/>
-      </c>
-      <c r="D58" s="16" t="inlineStr">
+      <c r="C60" s="65">
+        <f>C58+C59</f>
+        <v/>
+      </c>
+      <c r="D60" s="16" t="inlineStr">
         <is>
           <t>Kas Akhir (Sama dengan Neraca 2024)</t>
         </is>
       </c>
-      <c r="G58" s="66">
-        <f>SUM(G49,G50,G51,G52,G53,G54,G55,G56,G57)</f>
-        <v/>
-      </c>
-      <c r="H58" s="41" t="inlineStr">
-        <is>
-          <t>Kas Bersih Diperoleh dari Aktivitas Pendanaan</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="28" t="n"/>
-      <c r="B59" s="28" t="inlineStr">
+      <c r="G60" s="66">
+        <f>SUM(G51,G52,G53,G54,G55,G56,G57,G58,G59)</f>
+        <v/>
+      </c>
+      <c r="H60" s="41" t="inlineStr">
+        <is>
+          <t>Kas Bersih Diperoleh dari (Digunakan untuk) Aktivitas Pendanaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="28" t="n"/>
+      <c r="B61" s="28" t="inlineStr">
         <is>
           <t>VERIFIKASI / CEK SELISIH DENGAN NERACA 2024</t>
         </is>
       </c>
-      <c r="C59" s="68">
-        <f>C58-'Neraca (Balance Sheet)'!B8</f>
-        <v/>
-      </c>
-      <c r="D59" s="28" t="inlineStr">
+      <c r="C61" s="68">
+        <f>C60-'Neraca (Balance Sheet)'!B8</f>
+        <v/>
+      </c>
+      <c r="D61" s="28" t="inlineStr">
         <is>
           <t>Harus 0 (Balance)</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="G60" s="66">
-        <f>G36+G46+G58</f>
-        <v/>
-      </c>
-      <c r="H60" s="41" t="inlineStr">
-        <is>
-          <t>KENAIKAN / (PENURUNAN) BERSIH KAS DAN SETARA KAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="G61" s="66">
-        <f>'Neraca (Balance Sheet)'!C8</f>
-        <v/>
-      </c>
-      <c r="H61" s="41" t="inlineStr">
-        <is>
-          <t>Kas dan Setara Kas Awal Tahun (31 Desember 2023)</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="G62" s="66">
-        <f>G60+G61</f>
+        <f>G37+G48+G60</f>
         <v/>
       </c>
       <c r="H62" s="41" t="inlineStr">
         <is>
-          <t>Kas dan Setara Kas Akhir Tahun (31 Desember 2024)</t>
+          <t>KENAIKAN / (PENURUNAN) BERSIH KAS DAN SETARA KAS</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="G63" s="66">
-        <f>G62-'Neraca (Balance Sheet)'!B8+(G62-C58)</f>
+        <f>'Neraca (Balance Sheet)'!C8</f>
         <v/>
       </c>
       <c r="H63" s="41" t="inlineStr">
         <is>
-          <t>Cek: Selisih dengan Neraca 2024 &amp; dengan Kertas Kerja (harus 0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="B66" s="69" t="inlineStr">
+          <t>Kas dan Setara Kas Awal Tahun (31 Desember 2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="G64" s="66">
+        <f>G62+G63</f>
+        <v/>
+      </c>
+      <c r="H64" s="41" t="inlineStr">
+        <is>
+          <t>Kas dan Setara Kas Akhir Tahun (31 Desember 2024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="G65" s="66">
+        <f>G64-'Neraca (Balance Sheet)'!B8+(G64-C60)</f>
+        <v/>
+      </c>
+      <c r="H65" s="41" t="inlineStr">
+        <is>
+          <t>Cek: Selisih dengan Neraca 2024 &amp; Kertas Kerja (harus 0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>DATA TAMBAHAN DARI LAPORAN AUDIT (INPUT)</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>Jumlah (Rp)</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>Sumber</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="B73" s="10" t="inlineStr">
+        <is>
+          <t>Laba penjualan properti investasi 2024</t>
+        </is>
+      </c>
+      <c r="C73" s="69" t="n">
+        <v>102866676017</v>
+      </c>
+      <c r="D73" s="10" t="inlineStr">
+        <is>
+          <t>Draft_Report_BJS_2025.doc - Laba Rugi: Laba penjualan properti investasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="B74" s="10" t="inlineStr">
+        <is>
+          <t>Penerimaan kas penjualan properti investasi 2024</t>
+        </is>
+      </c>
+      <c r="C74" s="69" t="n">
+        <v>145577800018</v>
+      </c>
+      <c r="D74" s="10" t="inlineStr">
+        <is>
+          <t>Draft_Report_BJS_2025.doc - Laporan Arus Kas: Penerimaan penjualan properti investasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="B75" s="10" t="inlineStr">
+        <is>
+          <t>Penyusutan properti investasi 2024</t>
+        </is>
+      </c>
+      <c r="C75" s="69" t="n">
+        <v>4369696822</v>
+      </c>
+      <c r="D75" s="10" t="inlineStr">
+        <is>
+          <t>Draft_Report_BJS_2025.doc - Catatan 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="B76" s="10" t="inlineStr">
+        <is>
+          <t>Penyusutan aset tetap (beban usaha) 2024</t>
+        </is>
+      </c>
+      <c r="C76" s="69" t="n">
+        <v>1330417350</v>
+      </c>
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>Draft_Report_BJS_2025.doc - Catatan 25</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="B77" s="10" t="inlineStr">
+        <is>
+          <t>Penyusutan dalam beban pokok pendapatan 2024</t>
+        </is>
+      </c>
+      <c r="C77" s="69" t="n">
+        <v>1714609384</v>
+      </c>
+      <c r="D77" s="10" t="inlineStr">
+        <is>
+          <t>Draft_Report_BJS_2025.doc - Catatan 23</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="B78" s="10" t="inlineStr">
+        <is>
+          <t>Penyusutan aset hak guna 2024</t>
+        </is>
+      </c>
+      <c r="C78" s="69" t="n">
+        <v>927627462</v>
+      </c>
+      <c r="D78" s="10" t="inlineStr">
+        <is>
+          <t>Draft_Report_BJS_2025.doc - Catatan 12/14 (mutasi aset hak guna)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="B79" s="10" t="inlineStr">
+        <is>
+          <t>Penambahan aset hak guna 2024 (non-kas, lawan liabilitas sewa)</t>
+        </is>
+      </c>
+      <c r="C79" s="69" t="n">
+        <v>1347872168</v>
+      </c>
+      <c r="D79" s="10" t="inlineStr">
+        <is>
+          <t>Draft_Report_BJS_2025.doc - Catatan 12/14 (mutasi liabilitas sewa)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="16" t="inlineStr">
+        <is>
+          <t>Total penyusutan &amp; amortisasi 2024</t>
+        </is>
+      </c>
+      <c r="C80" s="65">
+        <f>SUM($C$75,$C$76,$C$77,$C$78)</f>
+        <v/>
+      </c>
+      <c r="D80" s="16" t="inlineStr">
+        <is>
+          <t>Dipakai di baris penyusutan</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="B81" s="70" t="inlineStr">
+        <is>
+          <t>Angka berwarna biru adalah input dari laporan audit; ubah jika laporan final berbeda.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="B83" s="71" t="inlineStr">
         <is>
           <t>Catatan:</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="B67" s="70" t="inlineStr">
-        <is>
-          <t>1. Sumber data: Neraca &amp; Laba Rugi 31-Des-2024 dari template.xlsx; 31-Des-2023 dari WS_Consol_PT_Bukit_Jaya_Semesta_2023.xlsx (sheet WBS WPL Consol, kolom CONSOLIDATED).</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="B68" s="70" t="inlineStr">
-        <is>
-          <t>2. Kenaikan Investment mengandung laba belum terealisasi PT Colorpak Indonesia Tbk (non-kas) yang dieliminasi terhadap ekuitas; nilainya:</t>
-        </is>
-      </c>
-      <c r="C68" s="64">
+    <row r="84">
+      <c r="B84" s="72" t="inlineStr">
+        <is>
+          <t>1. Sumber: Neraca &amp; Laba Rugi 2024 dari Draft_Report_BJS_2025.doc (disajikan kembali); 2023 dari WS_Consol_PT_Bukit_Jaya_Semesta_2023.xlsx (WBS WPL Consol), dicocokkan dengan Catatan 4 laporan audit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="72" t="inlineStr">
+        <is>
+          <t>2. Kenaikan Investment mengandung perubahan nilai wajar PT Colorpak Indonesia Tbk (non-kas) yang dieliminasi terhadap ekuitas; nilainya:</t>
+        </is>
+      </c>
+      <c r="C85" s="64">
         <f>-'Neraca (Balance Sheet)'!D60</f>
         <v/>
       </c>
     </row>
-    <row r="69">
-      <c r="B69" s="70" t="inlineStr">
-        <is>
-          <t>3. Penyesuaian saldo laba = Selisih Saldo Laba di Neraca dikurangi Laba Komprehensif Mayoritas di Laba Rugi (idealnya 0 / pembulatan).</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="70" t="inlineStr">
-        <is>
-          <t>4. Arus kas tahun 2023 tidak disusun karena file sumber tidak memuat Neraca 31-Des-2022 (kolom tahun pembanding bernilai 0).</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="B71" s="70" t="inlineStr">
-        <is>
-          <t>5. File SalesByOrderStatus (order Sep-2026) tidak digunakan: periode &amp; entitasnya di luar laporan konsolidasi 2024-2023.</t>
+    <row r="86">
+      <c r="B86" s="72" t="inlineStr">
+        <is>
+          <t>3. Penjualan properti investasi 2024: laba 102,87 M dikeluarkan dari operasi; penerimaan kas 145,58 M disajikan di investasi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="B87" s="72" t="inlineStr">
+        <is>
+          <t>4. Penambahan aset hak guna (sewa baru) tidak melibatkan kas, sehingga dikeluarkan dari perolehan aset dan dari liabilitas sewa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="72" t="inlineStr">
+        <is>
+          <t>5. Laporan arus kas di Draft_Report_BJS_2025.doc adalah versi entitas induk sebelum penyajian kembali (kas akhir 21,72 M), sehingga tidak dipakai untuk konsolidasian.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="72" t="inlineStr">
+        <is>
+          <t>6. Arus kas 2023 tidak disusun karena sumber tidak memuat Neraca konsolidasian 31-Des-2022.</t>
         </is>
       </c>
     </row>
@@ -2300,14 +2520,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="4"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
@@ -2354,7 +2575,12 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Referensi 2023 (WBS WPL Consol)</t>
+          <t>Pos di Laporan Audit (Draft Report BJS 2025)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Referensi WS Consol 2023</t>
         </is>
       </c>
     </row>
@@ -2384,19 +2610,24 @@
           <t>Kas kecil</t>
         </is>
       </c>
-      <c r="B8" s="71" t="n">
+      <c r="B8" s="73" t="n">
         <v>49663124528</v>
       </c>
-      <c r="C8" s="71" t="n">
+      <c r="C8" s="73" t="n">
         <v>24203301123</v>
       </c>
-      <c r="D8" s="71">
+      <c r="D8" s="73">
         <f>C8-B8</f>
         <v/>
       </c>
-      <c r="E8" s="72" t="inlineStr">
-        <is>
-          <t>Baris 40 Total Kas &amp; Setara Kas</t>
+      <c r="E8" s="74" t="inlineStr">
+        <is>
+          <t>Kas dan bank</t>
+        </is>
+      </c>
+      <c r="F8" s="74" t="inlineStr">
+        <is>
+          <t>Baris 40</t>
         </is>
       </c>
     </row>
@@ -2406,17 +2637,22 @@
           <t>Restricted Cash</t>
         </is>
       </c>
-      <c r="B9" s="71" t="n">
+      <c r="B9" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="71" t="n">
+      <c r="C9" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="71">
+      <c r="D9" s="73">
         <f>C9-B9</f>
         <v/>
       </c>
-      <c r="E9" s="72" t="inlineStr">
+      <c r="E9" s="74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F9" s="74" t="inlineStr">
         <is>
           <t>Baris 42</t>
         </is>
@@ -2428,19 +2664,24 @@
           <t>Piutang usaha - bersih</t>
         </is>
       </c>
-      <c r="B10" s="71" t="n">
+      <c r="B10" s="73" t="n">
         <v>12963459099</v>
       </c>
-      <c r="C10" s="71" t="n">
+      <c r="C10" s="73" t="n">
         <v>5078206703</v>
       </c>
-      <c r="D10" s="71">
+      <c r="D10" s="73">
         <f>C10-B10</f>
         <v/>
       </c>
-      <c r="E10" s="72" t="inlineStr">
-        <is>
-          <t>Baris 117 (Pihak ketiga 105 + berelasi 113)</t>
+      <c r="E10" s="74" t="inlineStr">
+        <is>
+          <t>Piutang usaha pihak ketiga + pihak berelasi</t>
+        </is>
+      </c>
+      <c r="F10" s="74" t="inlineStr">
+        <is>
+          <t>Baris 117</t>
         </is>
       </c>
     </row>
@@ -2450,17 +2691,22 @@
           <t>Piutang lain-lain - pihak ketiga</t>
         </is>
       </c>
-      <c r="B11" s="71" t="n">
+      <c r="B11" s="73" t="n">
         <v>2088735497</v>
       </c>
-      <c r="C11" s="71" t="n">
+      <c r="C11" s="73" t="n">
         <v>3433169417</v>
       </c>
-      <c r="D11" s="71">
+      <c r="D11" s="73">
         <f>C11-B11</f>
         <v/>
       </c>
-      <c r="E11" s="72" t="inlineStr">
+      <c r="E11" s="74" t="inlineStr">
+        <is>
+          <t>Piutang pembiayaan modal kerja + piutang lain-lain pihak ketiga</t>
+        </is>
+      </c>
+      <c r="F11" s="74" t="inlineStr">
         <is>
           <t>Baris 127</t>
         </is>
@@ -2472,17 +2718,22 @@
           <t>Piutang lain-lain - pihak berelasi</t>
         </is>
       </c>
-      <c r="B12" s="71" t="n">
+      <c r="B12" s="73" t="n">
         <v>13543645093</v>
       </c>
-      <c r="C12" s="71" t="n">
+      <c r="C12" s="73" t="n">
         <v>8950000000</v>
       </c>
-      <c r="D12" s="71">
+      <c r="D12" s="73">
         <f>C12-B12</f>
         <v/>
       </c>
-      <c r="E12" s="72" t="inlineStr">
+      <c r="E12" s="74" t="inlineStr">
+        <is>
+          <t>Piutang lain-lain pihak berelasi</t>
+        </is>
+      </c>
+      <c r="F12" s="74" t="inlineStr">
         <is>
           <t>Baris 134</t>
         </is>
@@ -2494,17 +2745,22 @@
           <t>Pajak dibayar di muka</t>
         </is>
       </c>
-      <c r="B13" s="71" t="n">
+      <c r="B13" s="73" t="n">
         <v>281571895</v>
       </c>
-      <c r="C13" s="71" t="n">
+      <c r="C13" s="73" t="n">
         <v>257219804</v>
       </c>
-      <c r="D13" s="71">
+      <c r="D13" s="73">
         <f>C13-B13</f>
         <v/>
       </c>
-      <c r="E13" s="72" t="inlineStr">
+      <c r="E13" s="74" t="inlineStr">
+        <is>
+          <t>Pajak dibayar di muka</t>
+        </is>
+      </c>
+      <c r="F13" s="74" t="inlineStr">
         <is>
           <t>Baris 144</t>
         </is>
@@ -2516,17 +2772,22 @@
           <t>Uang muka</t>
         </is>
       </c>
-      <c r="B14" s="71" t="n">
+      <c r="B14" s="73" t="n">
         <v>327111435</v>
       </c>
-      <c r="C14" s="71" t="n">
+      <c r="C14" s="73" t="n">
         <v>1383039636</v>
       </c>
-      <c r="D14" s="71">
+      <c r="D14" s="73">
         <f>C14-B14</f>
         <v/>
       </c>
-      <c r="E14" s="72" t="inlineStr">
+      <c r="E14" s="74" t="inlineStr">
+        <is>
+          <t>Uang muka dan biaya dibayar di muka (bagian uang muka)</t>
+        </is>
+      </c>
+      <c r="F14" s="74" t="inlineStr">
         <is>
           <t>Baris 159</t>
         </is>
@@ -2538,17 +2799,22 @@
           <t>Persediaaan</t>
         </is>
       </c>
-      <c r="B15" s="71" t="n">
+      <c r="B15" s="73" t="n">
         <v>3825027103</v>
       </c>
-      <c r="C15" s="71" t="n">
+      <c r="C15" s="73" t="n">
         <v>1434622080</v>
       </c>
-      <c r="D15" s="71">
+      <c r="D15" s="73">
         <f>C15-B15</f>
         <v/>
       </c>
-      <c r="E15" s="72" t="inlineStr">
+      <c r="E15" s="74" t="inlineStr">
+        <is>
+          <t>Persediaan</t>
+        </is>
+      </c>
+      <c r="F15" s="74" t="inlineStr">
         <is>
           <t>Baris 187</t>
         </is>
@@ -2560,17 +2826,22 @@
           <t>Biaya dibayar dimuka</t>
         </is>
       </c>
-      <c r="B16" s="71" t="n">
+      <c r="B16" s="73" t="n">
         <v>1171842931</v>
       </c>
-      <c r="C16" s="71" t="n">
+      <c r="C16" s="73" t="n">
         <v>960221120</v>
       </c>
-      <c r="D16" s="71">
+      <c r="D16" s="73">
         <f>C16-B16</f>
         <v/>
       </c>
-      <c r="E16" s="72" t="inlineStr">
+      <c r="E16" s="74" t="inlineStr">
+        <is>
+          <t>Uang muka dan biaya dibayar di muka (bagian biaya dibayar di muka)</t>
+        </is>
+      </c>
+      <c r="F16" s="74" t="inlineStr">
         <is>
           <t>Baris 151</t>
         </is>
@@ -2582,17 +2853,22 @@
           <t>Persediaan bilogis</t>
         </is>
       </c>
-      <c r="B17" s="71" t="n">
+      <c r="B17" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="C17" s="71" t="n">
+      <c r="C17" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="71">
+      <c r="D17" s="73">
         <f>C17-B17</f>
         <v/>
       </c>
-      <c r="E17" s="72" t="inlineStr">
+      <c r="E17" s="74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F17" s="74" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2604,15 +2880,15 @@
           <t>TOTAL ASET LANCAR</t>
         </is>
       </c>
-      <c r="B18" s="73">
+      <c r="B18" s="75">
         <f>SUM(B8:B17)</f>
         <v/>
       </c>
-      <c r="C18" s="73">
+      <c r="C18" s="75">
         <f>SUM(C8:C17)</f>
         <v/>
       </c>
-      <c r="D18" s="73">
+      <c r="D18" s="75">
         <f>C18-B18</f>
         <v/>
       </c>
@@ -2649,19 +2925,24 @@
           <t xml:space="preserve">  Harga perolehan</t>
         </is>
       </c>
-      <c r="B22" s="71" t="n">
+      <c r="B22" s="73" t="n">
         <v>604765019086</v>
       </c>
-      <c r="C22" s="71" t="n">
+      <c r="C22" s="73" t="n">
         <v>537668235420</v>
       </c>
-      <c r="D22" s="71">
+      <c r="D22" s="73">
         <f>C22-B22</f>
         <v/>
       </c>
-      <c r="E22" s="72" t="inlineStr">
-        <is>
-          <t>Baris 275 (termasuk properti investasi)</t>
+      <c r="E22" s="74" t="inlineStr">
+        <is>
+          <t>Properti investasi + aset tetap + aset hak guna + aset tak berwujud (biaya perolehan)</t>
+        </is>
+      </c>
+      <c r="F22" s="74" t="inlineStr">
+        <is>
+          <t>Baris 275</t>
         </is>
       </c>
     </row>
@@ -2671,17 +2952,22 @@
           <t xml:space="preserve">  Penyusutan</t>
         </is>
       </c>
-      <c r="B23" s="71" t="n">
+      <c r="B23" s="73" t="n">
         <v>-38841748680</v>
       </c>
-      <c r="C23" s="71" t="n">
+      <c r="C23" s="73" t="n">
         <v>-39986601780</v>
       </c>
-      <c r="D23" s="71">
+      <c r="D23" s="73">
         <f>C23-B23</f>
         <v/>
       </c>
-      <c r="E23" s="72" t="inlineStr">
+      <c r="E23" s="74" t="inlineStr">
+        <is>
+          <t>Akumulasi penyusutan atas pos di atas</t>
+        </is>
+      </c>
+      <c r="F23" s="74" t="inlineStr">
         <is>
           <t>Baris 296</t>
         </is>
@@ -2693,15 +2979,15 @@
           <t>Net Book Value</t>
         </is>
       </c>
-      <c r="B24" s="71">
+      <c r="B24" s="73">
         <f>SUM(B22:B23)</f>
         <v/>
       </c>
-      <c r="C24" s="71">
+      <c r="C24" s="73">
         <f>SUM(C22:C23)</f>
         <v/>
       </c>
-      <c r="D24" s="71">
+      <c r="D24" s="73">
         <f>C24-B24</f>
         <v/>
       </c>
@@ -2712,17 +2998,22 @@
           <t>Uang Muka Pembelian Aset Tetap</t>
         </is>
       </c>
-      <c r="B25" s="71" t="n">
+      <c r="B25" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="C25" s="71" t="n">
+      <c r="C25" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="D25" s="71">
+      <c r="D25" s="73">
         <f>C25-B25</f>
         <v/>
       </c>
-      <c r="E25" s="72" t="inlineStr">
+      <c r="E25" s="74" t="inlineStr">
+        <is>
+          <t>Uang muka pembelian tanah (2025)</t>
+        </is>
+      </c>
+      <c r="F25" s="74" t="inlineStr">
         <is>
           <t>Baris 302</t>
         </is>
@@ -2734,17 +3025,22 @@
           <t>Estimasi klaim pajak</t>
         </is>
       </c>
-      <c r="B26" s="71" t="n">
+      <c r="B26" s="73" t="n">
         <v>75307299</v>
       </c>
-      <c r="C26" s="71" t="n">
+      <c r="C26" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="D26" s="71">
+      <c r="D26" s="73">
         <f>C26-B26</f>
         <v/>
       </c>
-      <c r="E26" s="72" t="inlineStr">
+      <c r="E26" s="74" t="inlineStr">
+        <is>
+          <t>Tagihan pajak penghasilan</t>
+        </is>
+      </c>
+      <c r="F26" s="74" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2756,17 +3052,22 @@
           <t>Piutang pihak berelasi</t>
         </is>
       </c>
-      <c r="B27" s="71" t="n">
+      <c r="B27" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="C27" s="71" t="n">
+      <c r="C27" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="D27" s="71">
+      <c r="D27" s="73">
         <f>C27-B27</f>
         <v/>
       </c>
-      <c r="E27" s="72" t="inlineStr">
+      <c r="E27" s="74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F27" s="74" t="inlineStr">
         <is>
           <t>Baris 308</t>
         </is>
@@ -2778,17 +3079,22 @@
           <t>Investment</t>
         </is>
       </c>
-      <c r="B28" s="71" t="n">
+      <c r="B28" s="73" t="n">
         <v>67404618000</v>
       </c>
-      <c r="C28" s="71" t="n">
+      <c r="C28" s="73" t="n">
         <v>65528008185</v>
       </c>
-      <c r="D28" s="71">
+      <c r="D28" s="73">
         <f>C28-B28</f>
         <v/>
       </c>
-      <c r="E28" s="72" t="inlineStr">
+      <c r="E28" s="74" t="inlineStr">
+        <is>
+          <t>Investasi saham (Catatan 11)</t>
+        </is>
+      </c>
+      <c r="F28" s="74" t="inlineStr">
         <is>
           <t>Baris 245</t>
         </is>
@@ -2800,17 +3106,22 @@
           <t>HTI</t>
         </is>
       </c>
-      <c r="B29" s="71" t="n">
+      <c r="B29" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="C29" s="71" t="n">
+      <c r="C29" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="D29" s="71">
+      <c r="D29" s="73">
         <f>C29-B29</f>
         <v/>
       </c>
-      <c r="E29" s="72" t="inlineStr">
+      <c r="E29" s="74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F29" s="74" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -2822,17 +3133,22 @@
           <t>Aset pajak tangguhan</t>
         </is>
       </c>
-      <c r="B30" s="71" t="n">
+      <c r="B30" s="73" t="n">
         <v>766214497</v>
       </c>
-      <c r="C30" s="71" t="n">
+      <c r="C30" s="73" t="n">
         <v>1625452428</v>
       </c>
-      <c r="D30" s="71">
+      <c r="D30" s="73">
         <f>C30-B30</f>
         <v/>
       </c>
-      <c r="E30" s="72" t="inlineStr">
+      <c r="E30" s="74" t="inlineStr">
+        <is>
+          <t>Aset pajak tangguhan</t>
+        </is>
+      </c>
+      <c r="F30" s="74" t="inlineStr">
         <is>
           <t>Baris 341</t>
         </is>
@@ -2844,17 +3160,22 @@
           <t>Tanaman Belum Menghasilkan - Bibit Durian</t>
         </is>
       </c>
-      <c r="B31" s="71" t="n">
+      <c r="B31" s="73" t="n">
         <v>318750000</v>
       </c>
-      <c r="C31" s="71" t="n">
+      <c r="C31" s="73" t="n">
         <v>318750000</v>
       </c>
-      <c r="D31" s="71">
+      <c r="D31" s="73">
         <f>C31-B31</f>
         <v/>
       </c>
-      <c r="E31" s="72" t="inlineStr">
+      <c r="E31" s="74" t="inlineStr">
+        <is>
+          <t>Goodwill</t>
+        </is>
+      </c>
+      <c r="F31" s="74" t="inlineStr">
         <is>
           <t>Baris 333</t>
         </is>
@@ -2866,17 +3187,22 @@
           <t>Aset lainnya</t>
         </is>
       </c>
-      <c r="B32" s="71" t="n">
+      <c r="B32" s="73" t="n">
         <v>427749144</v>
       </c>
-      <c r="C32" s="71" t="n">
+      <c r="C32" s="73" t="n">
         <v>50000000</v>
       </c>
-      <c r="D32" s="71">
+      <c r="D32" s="73">
         <f>C32-B32</f>
         <v/>
       </c>
-      <c r="E32" s="72" t="inlineStr">
+      <c r="E32" s="74" t="inlineStr">
+        <is>
+          <t>Uang jaminan</t>
+        </is>
+      </c>
+      <c r="F32" s="74" t="inlineStr">
         <is>
           <t>Baris 346</t>
         </is>
@@ -2888,15 +3214,15 @@
           <t>TOTAL ASET TIDAK LANCAR</t>
         </is>
       </c>
-      <c r="B33" s="73">
+      <c r="B33" s="75">
         <f>B24+SUM(B25:B32)</f>
         <v/>
       </c>
-      <c r="C33" s="73">
+      <c r="C33" s="75">
         <f>C24+SUM(C25:C32)</f>
         <v/>
       </c>
-      <c r="D33" s="73">
+      <c r="D33" s="75">
         <f>C33-B33</f>
         <v/>
       </c>
@@ -2907,15 +3233,15 @@
           <t>TOTAL ASET</t>
         </is>
       </c>
-      <c r="B34" s="74">
+      <c r="B34" s="76">
         <f>B18+B33</f>
         <v/>
       </c>
-      <c r="C34" s="74">
+      <c r="C34" s="76">
         <f>C18+C33</f>
         <v/>
       </c>
-      <c r="D34" s="74">
+      <c r="D34" s="76">
         <f>C34-B34</f>
         <v/>
       </c>
@@ -2952,17 +3278,22 @@
           <t>Utang bank</t>
         </is>
       </c>
-      <c r="B38" s="71" t="n">
+      <c r="B38" s="73" t="n">
         <v>5850000000</v>
       </c>
-      <c r="C38" s="71" t="n">
+      <c r="C38" s="73" t="n">
         <v>17500000000</v>
       </c>
-      <c r="D38" s="71">
+      <c r="D38" s="73">
         <f>C38-B38</f>
         <v/>
       </c>
-      <c r="E38" s="72" t="inlineStr">
+      <c r="E38" s="74" t="inlineStr">
+        <is>
+          <t>Utang bank - bagian jangka pendek</t>
+        </is>
+      </c>
+      <c r="F38" s="74" t="inlineStr">
         <is>
           <t>Baris 367</t>
         </is>
@@ -2974,17 +3305,22 @@
           <t>Utang usaha</t>
         </is>
       </c>
-      <c r="B39" s="71" t="n">
+      <c r="B39" s="73" t="n">
         <v>5017737008</v>
       </c>
-      <c r="C39" s="71" t="n">
+      <c r="C39" s="73" t="n">
         <v>505654243</v>
       </c>
-      <c r="D39" s="71">
+      <c r="D39" s="73">
         <f>C39-B39</f>
         <v/>
       </c>
-      <c r="E39" s="72" t="inlineStr">
+      <c r="E39" s="74" t="inlineStr">
+        <is>
+          <t>Utang usaha pihak ketiga + pihak berelasi</t>
+        </is>
+      </c>
+      <c r="F39" s="74" t="inlineStr">
         <is>
           <t>Baris 411</t>
         </is>
@@ -2996,17 +3332,22 @@
           <t>Utang Pajak</t>
         </is>
       </c>
-      <c r="B40" s="71" t="n">
+      <c r="B40" s="73" t="n">
         <v>17506015406</v>
       </c>
-      <c r="C40" s="71" t="n">
+      <c r="C40" s="73" t="n">
         <v>1114165636</v>
       </c>
-      <c r="D40" s="71">
+      <c r="D40" s="73">
         <f>C40-B40</f>
         <v/>
       </c>
-      <c r="E40" s="72" t="inlineStr">
+      <c r="E40" s="74" t="inlineStr">
+        <is>
+          <t>Utang pajak</t>
+        </is>
+      </c>
+      <c r="F40" s="74" t="inlineStr">
         <is>
           <t>Baris 464</t>
         </is>
@@ -3018,17 +3359,22 @@
           <t>Uang muka penjualan</t>
         </is>
       </c>
-      <c r="B41" s="71" t="n">
+      <c r="B41" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="C41" s="71" t="n">
+      <c r="C41" s="73" t="n">
         <v>648000000</v>
       </c>
-      <c r="D41" s="71">
+      <c r="D41" s="73">
         <f>C41-B41</f>
         <v/>
       </c>
-      <c r="E41" s="72" t="inlineStr">
+      <c r="E41" s="74" t="inlineStr">
+        <is>
+          <t>Pendapatan diterima dimuka</t>
+        </is>
+      </c>
+      <c r="F41" s="74" t="inlineStr">
         <is>
           <t>Baris 469</t>
         </is>
@@ -3040,17 +3386,22 @@
           <t>Biaya masih harus dibayar</t>
         </is>
       </c>
-      <c r="B42" s="71" t="n">
+      <c r="B42" s="73" t="n">
         <v>1618002579</v>
       </c>
-      <c r="C42" s="71" t="n">
+      <c r="C42" s="73" t="n">
         <v>2010524052</v>
       </c>
-      <c r="D42" s="71">
+      <c r="D42" s="73">
         <f>C42-B42</f>
         <v/>
       </c>
-      <c r="E42" s="72" t="inlineStr">
+      <c r="E42" s="74" t="inlineStr">
+        <is>
+          <t>Beban masih harus dibayar</t>
+        </is>
+      </c>
+      <c r="F42" s="74" t="inlineStr">
         <is>
           <t>Baris 449</t>
         </is>
@@ -3062,17 +3413,22 @@
           <t>Imbalan kerja janga pendek</t>
         </is>
       </c>
-      <c r="B43" s="71" t="n">
+      <c r="B43" s="73" t="n">
         <v>357242000</v>
       </c>
-      <c r="C43" s="71" t="n">
+      <c r="C43" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="D43" s="71">
+      <c r="D43" s="73">
         <f>C43-B43</f>
         <v/>
       </c>
-      <c r="E43" s="72" t="inlineStr">
+      <c r="E43" s="74" t="inlineStr">
+        <is>
+          <t>Liabilitas imbalan kerja - bagian jangka pendek</t>
+        </is>
+      </c>
+      <c r="F43" s="74" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3084,17 +3440,22 @@
           <t>Utang lain-lain - pihak ketiga</t>
         </is>
       </c>
-      <c r="B44" s="71" t="n">
+      <c r="B44" s="73" t="n">
         <v>1293050662</v>
       </c>
-      <c r="C44" s="71" t="n">
+      <c r="C44" s="73" t="n">
         <v>2179697795</v>
       </c>
-      <c r="D44" s="71">
+      <c r="D44" s="73">
         <f>C44-B44</f>
         <v/>
       </c>
-      <c r="E44" s="72" t="inlineStr">
+      <c r="E44" s="74" t="inlineStr">
+        <is>
+          <t>Utang lain-lain pihak ketiga</t>
+        </is>
+      </c>
+      <c r="F44" s="74" t="inlineStr">
         <is>
           <t>Baris 419</t>
         </is>
@@ -3106,17 +3467,22 @@
           <t>Utang lain-lain - pihak berelasi</t>
         </is>
       </c>
-      <c r="B45" s="71" t="n">
+      <c r="B45" s="73" t="n">
         <v>2279605092</v>
       </c>
-      <c r="C45" s="71" t="n">
+      <c r="C45" s="73" t="n">
         <v>7644345919</v>
       </c>
-      <c r="D45" s="71">
+      <c r="D45" s="73">
         <f>C45-B45</f>
         <v/>
       </c>
-      <c r="E45" s="72" t="inlineStr">
+      <c r="E45" s="74" t="inlineStr">
+        <is>
+          <t>Utang lain-lain pihak berelasi</t>
+        </is>
+      </c>
+      <c r="F45" s="74" t="inlineStr">
         <is>
           <t>Baris 432</t>
         </is>
@@ -3128,17 +3494,22 @@
           <t>Utang pihak berelasi - jangka pendek</t>
         </is>
       </c>
-      <c r="B46" s="71" t="n">
+      <c r="B46" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="C46" s="71" t="n">
+      <c r="C46" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="D46" s="71">
+      <c r="D46" s="73">
         <f>C46-B46</f>
         <v/>
       </c>
-      <c r="E46" s="72" t="inlineStr">
+      <c r="E46" s="74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F46" s="74" t="inlineStr">
         <is>
           <t>Baris 476</t>
         </is>
@@ -3150,17 +3521,22 @@
           <t>Liabilitas sewa</t>
         </is>
       </c>
-      <c r="B47" s="71" t="n">
+      <c r="B47" s="73" t="n">
         <v>1106759005</v>
       </c>
-      <c r="C47" s="71" t="n">
+      <c r="C47" s="73" t="n">
         <v>811931047</v>
       </c>
-      <c r="D47" s="71">
+      <c r="D47" s="73">
         <f>C47-B47</f>
         <v/>
       </c>
-      <c r="E47" s="72" t="inlineStr">
+      <c r="E47" s="74" t="inlineStr">
+        <is>
+          <t>Liabilitas sewa - bagian jangka pendek</t>
+        </is>
+      </c>
+      <c r="F47" s="74" t="inlineStr">
         <is>
           <t>Baris 474</t>
         </is>
@@ -3172,15 +3548,15 @@
           <t>TOTAL LIABILITAS JANGKA PENDEK</t>
         </is>
       </c>
-      <c r="B48" s="73">
+      <c r="B48" s="75">
         <f>SUM(B38:B47)</f>
         <v/>
       </c>
-      <c r="C48" s="73">
+      <c r="C48" s="75">
         <f>SUM(C38:C47)</f>
         <v/>
       </c>
-      <c r="D48" s="73">
+      <c r="D48" s="75">
         <f>C48-B48</f>
         <v/>
       </c>
@@ -3207,17 +3583,22 @@
           <t>Imbalan kerja karyawan</t>
         </is>
       </c>
-      <c r="B51" s="71" t="n">
+      <c r="B51" s="73" t="n">
         <v>3901933524</v>
       </c>
-      <c r="C51" s="71" t="n">
+      <c r="C51" s="73" t="n">
         <v>2899127504</v>
       </c>
-      <c r="D51" s="71">
+      <c r="D51" s="73">
         <f>C51-B51</f>
         <v/>
       </c>
-      <c r="E51" s="72" t="inlineStr">
+      <c r="E51" s="74" t="inlineStr">
+        <is>
+          <t>Liabilitas imbalan kerja</t>
+        </is>
+      </c>
+      <c r="F51" s="74" t="inlineStr">
         <is>
           <t>Baris 489</t>
         </is>
@@ -3229,17 +3610,22 @@
           <t>Utang bank</t>
         </is>
       </c>
-      <c r="B52" s="71" t="n">
+      <c r="B52" s="73" t="n">
         <v>70268000000</v>
       </c>
-      <c r="C52" s="71" t="n">
+      <c r="C52" s="73" t="n">
         <v>52987000000</v>
       </c>
-      <c r="D52" s="71">
+      <c r="D52" s="73">
         <f>C52-B52</f>
         <v/>
       </c>
-      <c r="E52" s="72" t="inlineStr">
+      <c r="E52" s="74" t="inlineStr">
+        <is>
+          <t>Utang bank - jangka panjang</t>
+        </is>
+      </c>
+      <c r="F52" s="74" t="inlineStr">
         <is>
           <t>Baris 486</t>
         </is>
@@ -3251,17 +3637,22 @@
           <t>Utang pihak berelasi</t>
         </is>
       </c>
-      <c r="B53" s="71" t="n">
-        <v>106524999999</v>
-      </c>
-      <c r="C53" s="71" t="n">
+      <c r="B53" s="73" t="n">
+        <v>106525000000</v>
+      </c>
+      <c r="C53" s="73" t="n">
         <v>185424812622</v>
       </c>
-      <c r="D53" s="71">
+      <c r="D53" s="73">
         <f>C53-B53</f>
         <v/>
       </c>
-      <c r="E53" s="72" t="inlineStr">
+      <c r="E53" s="74" t="inlineStr">
+        <is>
+          <t>Utang pihak berelasi</t>
+        </is>
+      </c>
+      <c r="F53" s="74" t="inlineStr">
         <is>
           <t>Baris 531</t>
         </is>
@@ -3273,17 +3664,22 @@
           <t>Liabilitas sewa</t>
         </is>
       </c>
-      <c r="B54" s="71" t="n">
+      <c r="B54" s="73" t="n">
         <v>311982223</v>
       </c>
-      <c r="C54" s="71" t="n">
+      <c r="C54" s="73" t="n">
         <v>121640061</v>
       </c>
-      <c r="D54" s="71">
+      <c r="D54" s="73">
         <f>C54-B54</f>
         <v/>
       </c>
-      <c r="E54" s="72" t="inlineStr">
+      <c r="E54" s="74" t="inlineStr">
+        <is>
+          <t>Liabilitas sewa - jangka panjang</t>
+        </is>
+      </c>
+      <c r="F54" s="74" t="inlineStr">
         <is>
           <t>Baris 536</t>
         </is>
@@ -3295,15 +3691,15 @@
           <t>TOTAL LIABILITAS JANGKA PANJANG</t>
         </is>
       </c>
-      <c r="B55" s="73">
+      <c r="B55" s="75">
         <f>SUM(B51:B54)</f>
         <v/>
       </c>
-      <c r="C55" s="73">
+      <c r="C55" s="75">
         <f>SUM(C51:C54)</f>
         <v/>
       </c>
-      <c r="D55" s="73">
+      <c r="D55" s="75">
         <f>C55-B55</f>
         <v/>
       </c>
@@ -3314,15 +3710,15 @@
           <t>TOTAL LIABILITAS</t>
         </is>
       </c>
-      <c r="B56" s="73">
+      <c r="B56" s="75">
         <f>B48+B55</f>
         <v/>
       </c>
-      <c r="C56" s="73">
+      <c r="C56" s="75">
         <f>C48+C55</f>
         <v/>
       </c>
-      <c r="D56" s="73">
+      <c r="D56" s="75">
         <f>C56-B56</f>
         <v/>
       </c>
@@ -3349,17 +3745,22 @@
           <t>Modal disetor</t>
         </is>
       </c>
-      <c r="B59" s="71" t="n">
+      <c r="B59" s="73" t="n">
         <v>20000000000</v>
       </c>
-      <c r="C59" s="71" t="n">
+      <c r="C59" s="73" t="n">
         <v>20000000000</v>
       </c>
-      <c r="D59" s="71">
+      <c r="D59" s="73">
         <f>C59-B59</f>
         <v/>
       </c>
-      <c r="E59" s="72" t="inlineStr">
+      <c r="E59" s="74" t="inlineStr">
+        <is>
+          <t>Modal saham</t>
+        </is>
+      </c>
+      <c r="F59" s="74" t="inlineStr">
         <is>
           <t>Baris 565</t>
         </is>
@@ -3371,17 +3772,22 @@
           <t>Laba/ (Rugi) belum terealisasi - PT Colorpak Indonesia Tbk</t>
         </is>
       </c>
-      <c r="B60" s="71" t="n">
+      <c r="B60" s="73" t="n">
         <v>11498752001</v>
       </c>
-      <c r="C60" s="71" t="n">
+      <c r="C60" s="73" t="n">
         <v>9792104501</v>
       </c>
-      <c r="D60" s="71">
+      <c r="D60" s="73">
         <f>C60-B60</f>
         <v/>
       </c>
-      <c r="E60" s="72" t="inlineStr">
+      <c r="E60" s="74" t="inlineStr">
+        <is>
+          <t>Perubahan nilai wajar investasi ekuitas yang belum terealisasi</t>
+        </is>
+      </c>
+      <c r="F60" s="74" t="inlineStr">
         <is>
           <t>Baris 573</t>
         </is>
@@ -3393,17 +3799,22 @@
           <t>Tambahan modal di setor</t>
         </is>
       </c>
-      <c r="B61" s="71" t="n">
+      <c r="B61" s="73" t="n">
         <v>8000000000</v>
       </c>
-      <c r="C61" s="71" t="n">
+      <c r="C61" s="73" t="n">
         <v>8000000000</v>
       </c>
-      <c r="D61" s="71">
+      <c r="D61" s="73">
         <f>C61-B61</f>
         <v/>
       </c>
-      <c r="E61" s="72" t="inlineStr">
+      <c r="E61" s="74" t="inlineStr">
+        <is>
+          <t>Tambahan modal disetor - pengampunan pajak</t>
+        </is>
+      </c>
+      <c r="F61" s="74" t="inlineStr">
         <is>
           <t>Baris 546</t>
         </is>
@@ -3415,17 +3826,22 @@
           <t>Stress</t>
         </is>
       </c>
-      <c r="B62" s="71" t="n">
+      <c r="B62" s="73" t="n">
         <v>256473449</v>
       </c>
-      <c r="C62" s="71" t="n">
+      <c r="C62" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="D62" s="71">
+      <c r="D62" s="73">
         <f>C62-B62</f>
         <v/>
       </c>
-      <c r="E62" s="72" t="inlineStr">
+      <c r="E62" s="74" t="inlineStr">
+        <is>
+          <t>Selisih transaksi perubahan saham anak</t>
+        </is>
+      </c>
+      <c r="F62" s="74" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3447,17 +3863,22 @@
           <t xml:space="preserve">  Beginning balance</t>
         </is>
       </c>
-      <c r="B64" s="71" t="n">
+      <c r="B64" s="73" t="n">
         <v>192833795710</v>
       </c>
-      <c r="C64" s="71" t="n">
+      <c r="C64" s="73" t="n">
         <v>187154813818</v>
       </c>
-      <c r="D64" s="71">
+      <c r="D64" s="73">
         <f>C64-B64</f>
         <v/>
       </c>
-      <c r="E64" s="72" t="inlineStr">
+      <c r="E64" s="74" t="inlineStr">
+        <is>
+          <t>Saldo laba awal</t>
+        </is>
+      </c>
+      <c r="F64" s="74" t="inlineStr">
         <is>
           <t>Baris 576</t>
         </is>
@@ -3469,17 +3890,22 @@
           <t xml:space="preserve">  Current earning</t>
         </is>
       </c>
-      <c r="B65" s="71" t="n">
+      <c r="B65" s="73" t="n">
         <v>115230255592</v>
       </c>
-      <c r="C65" s="71" t="n">
+      <c r="C65" s="73" t="n">
         <v>5678981891</v>
       </c>
-      <c r="D65" s="71">
+      <c r="D65" s="73">
         <f>C65-B65</f>
         <v/>
       </c>
-      <c r="E65" s="72" t="inlineStr">
+      <c r="E65" s="74" t="inlineStr">
+        <is>
+          <t>Laba komprehensif diatribusikan ke pemilik entitas induk</t>
+        </is>
+      </c>
+      <c r="F65" s="74" t="inlineStr">
         <is>
           <t>Baris 592</t>
         </is>
@@ -3491,15 +3917,15 @@
           <t xml:space="preserve">  Ending balance</t>
         </is>
       </c>
-      <c r="B66" s="71">
+      <c r="B66" s="73">
         <f>SUM(B64:B65)</f>
         <v/>
       </c>
-      <c r="C66" s="71">
+      <c r="C66" s="73">
         <f>SUM(C64:C65)</f>
         <v/>
       </c>
-      <c r="D66" s="71">
+      <c r="D66" s="73">
         <f>C66-B66</f>
         <v/>
       </c>
@@ -3510,17 +3936,22 @@
           <t>NCI</t>
         </is>
       </c>
-      <c r="B67" s="71" t="n">
+      <c r="B67" s="73" t="n">
         <v>154925822676</v>
       </c>
-      <c r="C67" s="71" t="n">
+      <c r="C67" s="73" t="n">
         <v>106430825047</v>
       </c>
-      <c r="D67" s="71">
+      <c r="D67" s="73">
         <f>C67-B67</f>
         <v/>
       </c>
-      <c r="E67" s="72" t="inlineStr">
+      <c r="E67" s="74" t="inlineStr">
+        <is>
+          <t>Kepentingan nonpengendali</t>
+        </is>
+      </c>
+      <c r="F67" s="74" t="inlineStr">
         <is>
           <t>Baris 550</t>
         </is>
@@ -3532,15 +3963,15 @@
           <t>TOTAL EKUITAS</t>
         </is>
       </c>
-      <c r="B68" s="73">
+      <c r="B68" s="75">
         <f>B59+B60+B61+B62+B66+B67</f>
         <v/>
       </c>
-      <c r="C68" s="73">
+      <c r="C68" s="75">
         <f>C59+C60+C61+C62+C66+C67</f>
         <v/>
       </c>
-      <c r="D68" s="73">
+      <c r="D68" s="75">
         <f>C68-B68</f>
         <v/>
       </c>
@@ -3551,59 +3982,93 @@
           <t>TOTAL LIABILITAS DAN EKUITAS</t>
         </is>
       </c>
-      <c r="B69" s="74">
+      <c r="B69" s="76">
         <f>B56+B68</f>
         <v/>
       </c>
-      <c r="C69" s="74">
+      <c r="C69" s="76">
         <f>C56+C68</f>
         <v/>
       </c>
-      <c r="D69" s="74">
+      <c r="D69" s="76">
         <f>C69-B69</f>
         <v/>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="75" t="inlineStr">
+      <c r="A71" s="77" t="inlineStr">
         <is>
           <t>Cek: Total Liabilitas &amp; Ekuitas - Total Aset (harus 0)</t>
         </is>
       </c>
-      <c r="B71" s="76">
+      <c r="B71" s="78">
         <f>B69-B34</f>
         <v/>
       </c>
-      <c r="C71" s="76">
+      <c r="C71" s="78">
         <f>C69-C34</f>
         <v/>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="75" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="77" t="inlineStr">
+        <is>
+          <t>Cek: Total Aset vs Laporan Audit</t>
+        </is>
+      </c>
+      <c r="B72" s="79">
+        <f>B34-718780426927</f>
+        <v/>
+      </c>
+      <c r="C72" s="79">
+        <f>C34-610903624136</f>
+        <v/>
+      </c>
+      <c r="E72" s="74" t="inlineStr">
+        <is>
+          <t>Jumlah aset per laporan audit: 718.780.426.927 (2024) dan 610.903.624.136 (2023)</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="80" t="inlineStr">
         <is>
           <t>Sumber data:</t>
         </is>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="77" t="inlineStr">
-        <is>
-          <t>• 31-Dec-24: template.xlsx, sheet Neraca kolom 31-Dec-24.</t>
-        </is>
-      </c>
-    </row>
     <row r="75">
-      <c r="A75" s="77" t="inlineStr">
-        <is>
-          <t>• 31-Dec-23: WS_Consol_PT_Bukit_Jaya_Semesta_2023.xlsx › 'WBS WPL Consol' kolom AH (CONSOLIDATED, Per Audit, 31-Des-2023).</t>
+      <c r="A75" s="70" t="inlineStr">
+        <is>
+          <t>• 31-Dec-24: Draft_Report_BJS_2025.doc - Laporan Posisi Keuangan Konsolidasian, kolom 2024 (disajikan kembali, Catatan 4); sama dengan kolom 31-Dec-24 pada Kertas Kerja Lengkap.</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="77" t="inlineStr">
-        <is>
-          <t>• Kolom "Selisih / Perubahan" = 2023 - 2024 (dipakai langsung oleh Kertas Kerja Cash Flow).</t>
+      <c r="A76" s="70" t="inlineStr">
+        <is>
+          <t>• 31-Dec-23: WS_Consol_PT_Bukit_Jaya_Semesta_2023.xlsx - sheet WBS WPL Consol kolom CONSOLIDATED (Per Audit); dicocokkan dengan kolom 2023 Draft_Report_BJS_2025.doc.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="70" t="inlineStr">
+        <is>
+          <t>• Harga perolehan &amp; penyusutan menggabungkan properti investasi, aset tetap, aset hak guna, dan aset tak berwujud (sesuai struktur template).</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="70" t="inlineStr">
+        <is>
+          <t>• Utang pihak berelasi 2024 memakai angka laporan audit 106.525.000.000 (template: 106.524.999.999), sehingga neraca 2024 balance tanpa selisih Rp1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="70" t="inlineStr">
+        <is>
+          <t>• Kolom "Selisih / Perubahan" = 2023 - 2024; dipakai langsung oleh Kertas Kerja Cash Flow.</t>
         </is>
       </c>
     </row>
@@ -3618,14 +4083,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="4"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="18.75" customHeight="1">
@@ -3672,7 +4138,12 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>Referensi 2023 (WBS WPL Consol)</t>
+          <t>Pos di Laporan Audit (Draft Report BJS 2025)</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Referensi WS Consol 2023</t>
         </is>
       </c>
     </row>
@@ -3682,17 +4153,22 @@
           <t>Penjualan</t>
         </is>
       </c>
-      <c r="B6" s="71" t="n">
+      <c r="B6" s="73" t="n">
         <v>92234715659</v>
       </c>
-      <c r="C6" s="71" t="n">
+      <c r="C6" s="73" t="n">
         <v>64437082090</v>
       </c>
-      <c r="D6" s="71">
+      <c r="D6" s="73">
         <f>C6-B6</f>
         <v/>
       </c>
-      <c r="E6" s="72" t="inlineStr">
+      <c r="E6" s="74" t="inlineStr">
+        <is>
+          <t>Pendapatan usaha</t>
+        </is>
+      </c>
+      <c r="F6" s="74" t="inlineStr">
         <is>
           <t>Baris 636</t>
         </is>
@@ -3704,17 +4180,22 @@
           <t>Beban Pokok Penjualan</t>
         </is>
       </c>
-      <c r="B7" s="71" t="n">
+      <c r="B7" s="73" t="n">
         <v>36602877527</v>
       </c>
-      <c r="C7" s="71" t="n">
+      <c r="C7" s="73" t="n">
         <v>17188336641</v>
       </c>
-      <c r="D7" s="71">
+      <c r="D7" s="73">
         <f>C7-B7</f>
         <v/>
       </c>
-      <c r="E7" s="72" t="inlineStr">
+      <c r="E7" s="74" t="inlineStr">
+        <is>
+          <t>Beban pokok pendapatan</t>
+        </is>
+      </c>
+      <c r="F7" s="74" t="inlineStr">
         <is>
           <t>Baris 701</t>
         </is>
@@ -3726,15 +4207,15 @@
           <t>Total Laba Kotor</t>
         </is>
       </c>
-      <c r="B8" s="73">
+      <c r="B8" s="75">
         <f>B6-B7</f>
         <v/>
       </c>
-      <c r="C8" s="73">
+      <c r="C8" s="75">
         <f>C6-C7</f>
         <v/>
       </c>
-      <c r="D8" s="73">
+      <c r="D8" s="75">
         <f>C8-B8</f>
         <v/>
       </c>
@@ -3761,17 +4242,22 @@
           <t xml:space="preserve">  Beban Usaha</t>
         </is>
       </c>
-      <c r="B11" s="71" t="n">
+      <c r="B11" s="73" t="n">
         <v>41184649120</v>
       </c>
-      <c r="C11" s="71" t="n">
+      <c r="C11" s="73" t="n">
         <v>46412531236</v>
       </c>
-      <c r="D11" s="71">
+      <c r="D11" s="73">
         <f>C11-B11</f>
         <v/>
       </c>
-      <c r="E11" s="72" t="inlineStr">
+      <c r="E11" s="74" t="inlineStr">
+        <is>
+          <t>Beban penjualan + beban usaha (2024: 12.939.191.881 + 28.245.457.239; 2023: 18.564.406.148 + 27.848.125.088)</t>
+        </is>
+      </c>
+      <c r="F11" s="74" t="inlineStr">
         <is>
           <t>Baris 773</t>
         </is>
@@ -3783,15 +4269,15 @@
           <t>Total Operating Expense</t>
         </is>
       </c>
-      <c r="B12" s="73">
+      <c r="B12" s="75">
         <f>B11</f>
         <v/>
       </c>
-      <c r="C12" s="73">
+      <c r="C12" s="75">
         <f>C11</f>
         <v/>
       </c>
-      <c r="D12" s="73">
+      <c r="D12" s="75">
         <f>C12-B12</f>
         <v/>
       </c>
@@ -3802,15 +4288,15 @@
           <t>Operating Income</t>
         </is>
       </c>
-      <c r="B13" s="73">
+      <c r="B13" s="75">
         <f>B8-B12</f>
         <v/>
       </c>
-      <c r="C13" s="73">
+      <c r="C13" s="75">
         <f>C8-C12</f>
         <v/>
       </c>
-      <c r="D13" s="73">
+      <c r="D13" s="75">
         <f>C13-B13</f>
         <v/>
       </c>
@@ -3837,19 +4323,24 @@
           <t xml:space="preserve">  Pendapatan Bunga</t>
         </is>
       </c>
-      <c r="B16" s="71" t="n">
+      <c r="B16" s="73" t="n">
         <v>10165418608</v>
       </c>
-      <c r="C16" s="71" t="n">
+      <c r="C16" s="73" t="n">
         <v>7264778074</v>
       </c>
-      <c r="D16" s="71">
+      <c r="D16" s="73">
         <f>C16-B16</f>
         <v/>
       </c>
-      <c r="E16" s="72" t="inlineStr">
-        <is>
-          <t>Baris 783 (pendapatan keuangan: bunga &amp; dividen)</t>
+      <c r="E16" s="74" t="inlineStr">
+        <is>
+          <t>Total pendapatan keuangan (dividen, jasa giro, bunga piutang modal kerja)</t>
+        </is>
+      </c>
+      <c r="F16" s="74" t="inlineStr">
+        <is>
+          <t>Baris 783</t>
         </is>
       </c>
     </row>
@@ -3859,17 +4350,22 @@
           <t xml:space="preserve">  Finance Expense</t>
         </is>
       </c>
-      <c r="B17" s="71" t="n">
+      <c r="B17" s="73" t="n">
         <v>-2443136567</v>
       </c>
-      <c r="C17" s="71" t="n">
+      <c r="C17" s="73" t="n">
         <v>-2116114767</v>
       </c>
-      <c r="D17" s="71">
+      <c r="D17" s="73">
         <f>C17-B17</f>
         <v/>
       </c>
-      <c r="E17" s="72" t="inlineStr">
+      <c r="E17" s="74" t="inlineStr">
+        <is>
+          <t>Total beban keuangan</t>
+        </is>
+      </c>
+      <c r="F17" s="74" t="inlineStr">
         <is>
           <t>Baris 794</t>
         </is>
@@ -3881,17 +4377,22 @@
           <t xml:space="preserve">  Lain-lain Net</t>
         </is>
       </c>
-      <c r="B18" s="71" t="n">
+      <c r="B18" s="73" t="n">
         <v>98866274584</v>
       </c>
-      <c r="C18" s="71" t="n">
+      <c r="C18" s="73" t="n">
         <v>312115524</v>
       </c>
-      <c r="D18" s="71">
+      <c r="D18" s="73">
         <f>C18-B18</f>
         <v/>
       </c>
-      <c r="E18" s="72" t="inlineStr">
+      <c r="E18" s="74" t="inlineStr">
+        <is>
+          <t>Total penghasilan (beban) lain-lain; 2024 termasuk laba penjualan properti investasi 102.866.676.017</t>
+        </is>
+      </c>
+      <c r="F18" s="74" t="inlineStr">
         <is>
           <t>Baris 821</t>
         </is>
@@ -3903,15 +4404,15 @@
           <t>Total Other Income (Expense)</t>
         </is>
       </c>
-      <c r="B19" s="73">
+      <c r="B19" s="75">
         <f>SUM(B16:B18)</f>
         <v/>
       </c>
-      <c r="C19" s="73">
+      <c r="C19" s="75">
         <f>SUM(C16:C18)</f>
         <v/>
       </c>
-      <c r="D19" s="73">
+      <c r="D19" s="75">
         <f>C19-B19</f>
         <v/>
       </c>
@@ -3922,15 +4423,15 @@
           <t>Income Before Tax</t>
         </is>
       </c>
-      <c r="B20" s="73">
+      <c r="B20" s="75">
         <f>B13+B19</f>
         <v/>
       </c>
-      <c r="C20" s="73">
+      <c r="C20" s="75">
         <f>C13+C19</f>
         <v/>
       </c>
-      <c r="D20" s="73">
+      <c r="D20" s="75">
         <f>C20-B20</f>
         <v/>
       </c>
@@ -3957,17 +4458,22 @@
           <t xml:space="preserve">  Tahun Berjalan</t>
         </is>
       </c>
-      <c r="B23" s="71" t="n">
+      <c r="B23" s="73" t="n">
         <v>-1696705500</v>
       </c>
-      <c r="C23" s="71" t="n">
+      <c r="C23" s="73" t="n">
         <v>-960889</v>
       </c>
-      <c r="D23" s="71">
+      <c r="D23" s="73">
         <f>C23-B23</f>
         <v/>
       </c>
-      <c r="E23" s="72" t="inlineStr">
+      <c r="E23" s="74" t="inlineStr">
+        <is>
+          <t>Beban pajak kini</t>
+        </is>
+      </c>
+      <c r="F23" s="74" t="inlineStr">
         <is>
           <t>Baris 833</t>
         </is>
@@ -3979,17 +4485,22 @@
           <t xml:space="preserve">  Ditangguhkan</t>
         </is>
       </c>
-      <c r="B24" s="71" t="n">
+      <c r="B24" s="73" t="n">
         <v>-1949871786</v>
       </c>
-      <c r="C24" s="71" t="n">
+      <c r="C24" s="73" t="n">
         <v>-1384371756</v>
       </c>
-      <c r="D24" s="71">
+      <c r="D24" s="73">
         <f>C24-B24</f>
         <v/>
       </c>
-      <c r="E24" s="72" t="inlineStr">
+      <c r="E24" s="74" t="inlineStr">
+        <is>
+          <t>Beban pajak tangguhan</t>
+        </is>
+      </c>
+      <c r="F24" s="74" t="inlineStr">
         <is>
           <t>Baris 834</t>
         </is>
@@ -4001,15 +4512,15 @@
           <t>Tax Expense</t>
         </is>
       </c>
-      <c r="B25" s="73">
+      <c r="B25" s="75">
         <f>SUM(B23:B24)</f>
         <v/>
       </c>
-      <c r="C25" s="73">
+      <c r="C25" s="75">
         <f>SUM(C23:C24)</f>
         <v/>
       </c>
-      <c r="D25" s="73">
+      <c r="D25" s="75">
         <f>C25-B25</f>
         <v/>
       </c>
@@ -4020,15 +4531,15 @@
           <t>Net Income (Laba Bersih)</t>
         </is>
       </c>
-      <c r="B26" s="74">
+      <c r="B26" s="76">
         <f>B20+B25</f>
         <v/>
       </c>
-      <c r="C26" s="74">
+      <c r="C26" s="76">
         <f>C20+C25</f>
         <v/>
       </c>
-      <c r="D26" s="74">
+      <c r="D26" s="76">
         <f>C26-B26</f>
         <v/>
       </c>
@@ -4046,17 +4557,22 @@
           <t>Selisih laba rugi aktuarial atas imbalan kerja</t>
         </is>
       </c>
-      <c r="B30" s="78" t="n">
+      <c r="B30" s="81" t="n">
         <v>-132361128</v>
       </c>
-      <c r="C30" s="78" t="n">
+      <c r="C30" s="81" t="n">
         <v>72787959</v>
       </c>
-      <c r="D30" s="79">
+      <c r="D30" s="82">
         <f>C30-B30</f>
         <v/>
       </c>
-      <c r="E30" s="72" t="inlineStr">
+      <c r="E30" s="74" t="inlineStr">
+        <is>
+          <t>Pengukuran kembali liabilitas imbalan pascakerja</t>
+        </is>
+      </c>
+      <c r="F30" s="74" t="inlineStr">
         <is>
           <t>Baris 847</t>
         </is>
@@ -4068,44 +4584,49 @@
           <t>Efek pajak terkait - imbalan kerja</t>
         </is>
       </c>
-      <c r="B31" s="80" t="n">
-        <v>29119448.28</v>
-      </c>
-      <c r="C31" s="80" t="n">
+      <c r="B31" s="83" t="n">
+        <v>29119448</v>
+      </c>
+      <c r="C31" s="83" t="n">
         <v>69583345</v>
       </c>
-      <c r="D31" s="81">
+      <c r="D31" s="84">
         <f>C31-B31</f>
         <v/>
       </c>
-      <c r="E31" s="72" t="inlineStr">
+      <c r="E31" s="74" t="inlineStr">
+        <is>
+          <t>Pajak penghasilan terkait</t>
+        </is>
+      </c>
+      <c r="F31" s="74" t="inlineStr">
         <is>
           <t>Baris 848</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="75" t="inlineStr">
+      <c r="A32" s="77" t="inlineStr">
         <is>
           <t>Total Penghasilan Komprehensif Lain</t>
         </is>
       </c>
-      <c r="B32" s="82">
+      <c r="B32" s="85">
         <f>SUM(B30:B31)</f>
         <v/>
       </c>
-      <c r="C32" s="82">
+      <c r="C32" s="85">
         <f>SUM(C30:C31)</f>
         <v/>
       </c>
-      <c r="D32" s="79">
+      <c r="D32" s="82">
         <f>C32-B32</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="82" t="n"/>
-      <c r="C33" s="82" t="n"/>
+      <c r="B33" s="85" t="n"/>
+      <c r="C33" s="85" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="58" t="inlineStr">
@@ -4113,15 +4634,15 @@
           <t>TOTAL PENGHASILAN KOMPREHENSIF LAIN</t>
         </is>
       </c>
-      <c r="B34" s="76">
+      <c r="B34" s="78">
         <f>B26+B32</f>
         <v/>
       </c>
-      <c r="C34" s="76">
+      <c r="C34" s="78">
         <f>C26+C32</f>
         <v/>
       </c>
-      <c r="D34" s="83">
+      <c r="D34" s="79">
         <f>C34-B34</f>
         <v/>
       </c>
@@ -4132,17 +4653,22 @@
           <t>NONCONTROLLING INEREST (PL)</t>
         </is>
       </c>
-      <c r="B36" s="84" t="n">
-        <v>2069518579.991412</v>
-      </c>
-      <c r="C36" s="84" t="n">
+      <c r="B36" s="86" t="n">
+        <v>2069518580</v>
+      </c>
+      <c r="C36" s="86" t="n">
         <v>-636305110</v>
       </c>
-      <c r="D36" s="85">
+      <c r="D36" s="87">
         <f>C36-B36</f>
         <v/>
       </c>
-      <c r="E36" s="72" t="inlineStr">
+      <c r="E36" s="74" t="inlineStr">
+        <is>
+          <t>Laba (rugi) tahun berjalan - kepentingan nonpengendali</t>
+        </is>
+      </c>
+      <c r="F36" s="74" t="inlineStr">
         <is>
           <t>Baris 854</t>
         </is>
@@ -4150,8 +4676,8 @@
     </row>
     <row r="37">
       <c r="A37" s="59" t="n"/>
-      <c r="B37" s="86" t="n"/>
-      <c r="C37" s="86" t="n"/>
+      <c r="B37" s="88" t="n"/>
+      <c r="C37" s="88" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="59" t="inlineStr">
@@ -4159,11 +4685,11 @@
           <t>TOTAL NETO TAHUN BERJALAN - Mayoritas</t>
         </is>
       </c>
-      <c r="B38" s="71">
+      <c r="B38" s="73">
         <f>B34-B36</f>
         <v/>
       </c>
-      <c r="C38" s="71">
+      <c r="C38" s="73">
         <f>C34-C36</f>
         <v/>
       </c>
@@ -4173,8 +4699,8 @@
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="71" t="n"/>
-      <c r="C39" s="71" t="n"/>
+      <c r="B39" s="73" t="n"/>
+      <c r="C39" s="73" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="32" t="inlineStr">
@@ -4182,8 +4708,8 @@
           <t>NONCONTROLLING INEREST (PL)</t>
         </is>
       </c>
-      <c r="B40" s="71" t="n"/>
-      <c r="C40" s="71" t="n"/>
+      <c r="B40" s="73" t="n"/>
+      <c r="C40" s="73" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="34" t="inlineStr">
@@ -4191,17 +4717,22 @@
           <t>OCI</t>
         </is>
       </c>
-      <c r="B41" s="71" t="n">
-        <v>-17753207.7550615</v>
-      </c>
-      <c r="C41" s="71" t="n">
+      <c r="B41" s="73" t="n">
+        <v>-17753208</v>
+      </c>
+      <c r="C41" s="73" t="n">
         <v>14557592</v>
       </c>
       <c r="D41" s="64">
         <f>C41-B41</f>
         <v/>
       </c>
-      <c r="E41" s="72" t="inlineStr">
+      <c r="E41" s="74" t="inlineStr">
+        <is>
+          <t>Bagian NCI atas OCI (2024 neto -13.847.501 = 2.055.671.079 - 2.069.518.580)</t>
+        </is>
+      </c>
+      <c r="F41" s="74" t="inlineStr">
         <is>
           <t>Baris 859</t>
         </is>
@@ -4213,102 +4744,134 @@
           <t>Pajak terkait</t>
         </is>
       </c>
-      <c r="B42" s="84" t="n">
-        <v>3905705.734433494</v>
-      </c>
-      <c r="C42" s="84" t="n">
+      <c r="B42" s="86" t="n">
+        <v>3905706</v>
+      </c>
+      <c r="C42" s="86" t="n">
         <v>-3202670</v>
       </c>
-      <c r="D42" s="85">
+      <c r="D42" s="87">
         <f>C42-B42</f>
         <v/>
       </c>
-      <c r="E42" s="72" t="inlineStr">
+      <c r="E42" s="74" t="inlineStr">
+        <is>
+          <t>Bagian NCI atas pajak OCI</t>
+        </is>
+      </c>
+      <c r="F42" s="74" t="inlineStr">
         <is>
           <t>Baris 860</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="75" t="inlineStr">
+      <c r="A43" s="77" t="inlineStr">
         <is>
           <t>Total NCI atas OCI</t>
         </is>
       </c>
-      <c r="B43" s="87">
+      <c r="B43" s="89">
         <f>SUM(B41:B42)</f>
         <v/>
       </c>
-      <c r="C43" s="87">
+      <c r="C43" s="89">
         <f>SUM(C41:C42)</f>
         <v/>
       </c>
-      <c r="D43" s="88">
+      <c r="D43" s="90">
         <f>C43-B43</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="B44" s="71" t="n"/>
-      <c r="C44" s="71" t="n"/>
+      <c r="B44" s="73" t="n"/>
+      <c r="C44" s="73" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="75" t="inlineStr">
+      <c r="A45" s="77" t="inlineStr">
         <is>
           <t>LABA KOMPREHENSIF - Mayoritas (Current Earning)</t>
         </is>
       </c>
-      <c r="B45" s="76">
+      <c r="B45" s="78">
         <f>B38-B43</f>
         <v/>
       </c>
-      <c r="C45" s="76">
+      <c r="C45" s="78">
         <f>C38-C43</f>
         <v/>
       </c>
-      <c r="D45" s="83">
+      <c r="D45" s="79">
         <f>C45-B45</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="75" t="inlineStr">
+      <c r="A48" s="77" t="inlineStr">
         <is>
           <t>Selisih Laba Bersih vs Laba Komprehensif Mayoritas</t>
         </is>
       </c>
-      <c r="B48" s="76">
+      <c r="B48" s="78">
         <f>B26-B45</f>
         <v/>
       </c>
-      <c r="C48" s="76">
+      <c r="C48" s="78">
         <f>C26-C45</f>
         <v/>
       </c>
-      <c r="D48" s="83">
+      <c r="D48" s="79">
         <f>C48-B48</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="75" t="inlineStr">
-        <is>
-          <t>Cek ke Neraca: Current Earning (Neraca) - Laba Komprehensif Mayoritas</t>
-        </is>
-      </c>
-      <c r="B50" s="83">
+      <c r="A50" s="77" t="inlineStr">
+        <is>
+          <t>Cek ke Neraca: Current Earning (Neraca) - Laba Komprehensif Mayoritas (±1 = pembulatan)</t>
+        </is>
+      </c>
+      <c r="B50" s="79">
         <f>'Neraca (Balance Sheet)'!B65-B45</f>
         <v/>
       </c>
-      <c r="C50" s="83">
+      <c r="C50" s="79">
         <f>'Neraca (Balance Sheet)'!C65-C45</f>
         <v/>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="77" t="inlineStr">
-        <is>
-          <t>Sumber data: 2024 dari template.xlsx (kolom 31-Dec-24); 2023 dari WS_Consol_PT_Bukit_Jaya_Semesta_2023.xlsx › 'WBS WPL Consol' kolom AH (CONSOLIDATED, Per Audit, 31-Des-2023).</t>
+    <row r="51">
+      <c r="A51" s="77" t="inlineStr">
+        <is>
+          <t>Cek ke Laporan Audit: Laba Neto Tahun Berjalan</t>
+        </is>
+      </c>
+      <c r="B51" s="79">
+        <f>B26-117389168351</f>
+        <v/>
+      </c>
+      <c r="C51" s="79">
+        <f>C26-4911660399</f>
+        <v/>
+      </c>
+      <c r="E51" s="74" t="inlineStr">
+        <is>
+          <t>Laba neto per laporan audit: 117.389.168.351 (2024); 4.911.660.399 (2023, Catatan 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="70" t="inlineStr">
+        <is>
+          <t>Sumber data: 2024 dari Draft_Report_BJS_2025.doc (Laporan Laba Rugi Konsolidasian, kolom 2024); 2023 dari WS_Consol_PT_Bukit_Jaya_Semesta_2023.xlsx (WBS WPL Consol) = Catatan 4 Draft_Report_BJS_2025.doc (setelah disajikan kembali).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="70" t="inlineStr">
+        <is>
+          <t>Catatan: di draft laporan, jumlah atribusi laba 2024 (115.262.514.196 + 2.069.518.580 = 117.332.032.777) selisih 57.135.574 dari laba neto 117.389.168.351; yang dipakai adalah angka laporan utama, yang cocok dengan saldo laba di neraca.</t>
         </is>
       </c>
     </row>

</xml_diff>